<commit_message>
création du design de la page d'accueil, 1ere version; JDT
</commit_message>
<xml_diff>
--- a/documentation/JDT-personal/Journal-de-Travail_NademoYosef.xlsx
+++ b/documentation/JDT-personal/Journal-de-Travail_NademoYosef.xlsx
@@ -8,10 +8,10 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pn25kdv\Documents\GitHub\Passion_lecture_FRONTEND\documentation\JDT-personal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D9ED2FB-99A7-4828-AE97-40177FA6689F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CB4517E-5C28-4306-AEDB-247810C57B34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="Mvap2W10CJFFJsnvkGXSiMLvpngxTMJbJsIKFe7Hzjn0XDcmjGuvBC2FjUCZ/hpRpUhUrG1T4kBlDAIo3yqmSQ==" workbookSaltValue="KXjgXOcsUZI/j7UgPKltzw==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
+    <workbookView xWindow="31215" yWindow="2175" windowWidth="21600" windowHeight="11385" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal de travail" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="34">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -140,6 +140,9 @@
   </si>
   <si>
     <t>création de GitHub repository, création d'une structure des dossier et fichier, mettre les fichiers nessaisers; création de Git Project</t>
+  </si>
+  <si>
+    <t>création du design de la page d'accueil, 1ere version</t>
   </si>
 </sst>
 </file>
@@ -1085,7 +1088,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0</c:v>
+                  <c:v>2.0833333333333332E-2</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>1.3888888888888888E-2</c:v>
@@ -2048,7 +2051,7 @@
       </c>
       <c r="C3" s="22" t="str">
         <f>INT(E4/1440)&amp;" jours "&amp;INT(MOD(E4/1440,1)*24)&amp;" heurs "&amp;INT(MOD(MOD(E4/1440,1)*24,1)*60)&amp;" minutes"</f>
-        <v>0 jours 1 heurs 10 minutes</v>
+        <v>0 jours 1 heurs 40 minutes</v>
       </c>
       <c r="D3" s="22"/>
       <c r="E3" s="3"/>
@@ -2067,11 +2070,11 @@
       </c>
       <c r="D4" s="22">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="E4" s="40">
         <f>SUM(C4:D4)</f>
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="7"/>
@@ -2186,15 +2189,23 @@
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A10" s="8" t="str">
+      <c r="A10" s="8">
         <f>IF(ISBLANK(B10),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B10))</f>
-        <v/>
-      </c>
-      <c r="B10" s="46"/>
+        <v>15</v>
+      </c>
+      <c r="B10" s="46">
+        <v>45755</v>
+      </c>
       <c r="C10" s="47"/>
-      <c r="D10" s="48"/>
-      <c r="E10" s="49"/>
-      <c r="F10" s="36"/>
+      <c r="D10" s="48">
+        <v>30</v>
+      </c>
+      <c r="E10" s="49" t="s">
+        <v>21</v>
+      </c>
+      <c r="F10" s="36" t="s">
+        <v>33</v>
+      </c>
       <c r="G10" s="55"/>
       <c r="M10" t="s">
         <v>5</v>
@@ -8718,7 +8729,7 @@
       </c>
       <c r="B10">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Analyse!C10,'Journal de travail'!$D$7:$D$532)</f>
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="C10" s="37" t="str">
         <f>'Journal de travail'!M14</f>
@@ -8726,7 +8737,7 @@
       </c>
       <c r="D10" s="33">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>2.0833333333333332E-2</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
@@ -8753,7 +8764,7 @@
       </c>
       <c r="D12" s="34">
         <f>SUM(D4:D11)</f>
-        <v>4.8611111111111112E-2</v>
+        <v>6.9444444444444448E-2</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
@@ -8990,6 +9001,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="be0d3259-a7ce-4623-88ec-81594dfcbc1c" xsi:nil="true"/>
@@ -8998,15 +9018,6 @@
     </lcf76f155ced4ddcb4097134ff3c332f>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -9029,6 +9040,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -9037,12 +9056,4 @@
     <ds:schemaRef ds:uri="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
dossier routes, avec une liste des routes, photo de liste des routes, et tableau des routes
</commit_message>
<xml_diff>
--- a/documentation/JDT-personal/Journal-de-Travail_NademoYosef.xlsx
+++ b/documentation/JDT-personal/Journal-de-Travail_NademoYosef.xlsx
@@ -8,10 +8,10 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pn25kdv\Documents\GitHub\Passion_lecture_FRONTEND\documentation\JDT-personal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6835FC5-0194-4D70-A69C-B9BB3F70E8CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15179ACD-243B-4EFE-A21E-4605C6F42EC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="Mvap2W10CJFFJsnvkGXSiMLvpngxTMJbJsIKFe7Hzjn0XDcmjGuvBC2FjUCZ/hpRpUhUrG1T4kBlDAIo3yqmSQ==" workbookSaltValue="KXjgXOcsUZI/j7UgPKltzw==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="31215" yWindow="2175" windowWidth="21600" windowHeight="11385" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal de travail" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="38">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -143,6 +143,18 @@
   </si>
   <si>
     <t>création du design de la page d'accueil, 1ere version</t>
+  </si>
+  <si>
+    <t>création du design de footer, 1ere version</t>
+  </si>
+  <si>
+    <t>création du design de la page d'accueil</t>
+  </si>
+  <si>
+    <t>construction du docker(création des fichiers .env, .yml, .dockerfile pour avoir l'environnement nécessaire au développement de l'application web.)</t>
+  </si>
+  <si>
+    <t>dossier routes, avec une liste des routes, photo de liste des routes, et tableau des routes</t>
   </si>
 </sst>
 </file>
@@ -1073,7 +1085,7 @@
                   <c:v>1.3888888888888888E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>3.4722222222222224E-2</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -1088,10 +1100,10 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1.3888888888888888E-2</c:v>
+                  <c:v>3.4722222222222224E-2</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1.3888888888888888E-2</c:v>
+                  <c:v>2.4305555555555556E-2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2051,7 +2063,7 @@
       </c>
       <c r="C3" s="22" t="str">
         <f>INT(E4/1440)&amp;" jours "&amp;INT(MOD(E4/1440,1)*24)&amp;" heurs "&amp;INT(MOD(MOD(E4/1440,1)*24,1)*60)&amp;" minutes"</f>
-        <v>0 jours 1 heurs 30 minutes</v>
+        <v>0 jours 3 heurs 4 minutes</v>
       </c>
       <c r="D3" s="22"/>
       <c r="E3" s="3"/>
@@ -2070,11 +2082,11 @@
       </c>
       <c r="D4" s="22">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>90</v>
+        <v>185</v>
       </c>
       <c r="E4" s="40">
         <f>SUM(C4:D4)</f>
-        <v>90</v>
+        <v>185</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="7"/>
@@ -2218,15 +2230,23 @@
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A11" s="16" t="str">
+      <c r="A11" s="16">
         <f>IF(ISBLANK(B11),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B11))</f>
-        <v/>
-      </c>
-      <c r="B11" s="50"/>
+        <v>15</v>
+      </c>
+      <c r="B11" s="50">
+        <v>45756</v>
+      </c>
       <c r="C11" s="51"/>
-      <c r="D11" s="52"/>
-      <c r="E11" s="53"/>
-      <c r="F11" s="36"/>
+      <c r="D11" s="52">
+        <v>15</v>
+      </c>
+      <c r="E11" s="53" t="s">
+        <v>21</v>
+      </c>
+      <c r="F11" s="36" t="s">
+        <v>35</v>
+      </c>
       <c r="G11" s="56"/>
       <c r="M11" t="s">
         <v>6</v>
@@ -2239,15 +2259,23 @@
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A12" s="8" t="str">
+      <c r="A12" s="8">
         <f>IF(ISBLANK(B12),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B12))</f>
-        <v/>
-      </c>
-      <c r="B12" s="46"/>
+        <v>15</v>
+      </c>
+      <c r="B12" s="46">
+        <v>45756</v>
+      </c>
       <c r="C12" s="47"/>
-      <c r="D12" s="48"/>
-      <c r="E12" s="49"/>
-      <c r="F12" s="36"/>
+      <c r="D12" s="48">
+        <v>15</v>
+      </c>
+      <c r="E12" s="49" t="s">
+        <v>21</v>
+      </c>
+      <c r="F12" s="36" t="s">
+        <v>34</v>
+      </c>
       <c r="G12" s="55"/>
       <c r="M12" t="s">
         <v>7</v>
@@ -2259,16 +2287,24 @@
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A13" s="16" t="str">
+    <row r="13" spans="1:15" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A13" s="16">
         <f>IF(ISBLANK(B13),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B13))</f>
-        <v/>
-      </c>
-      <c r="B13" s="50"/>
+        <v>15</v>
+      </c>
+      <c r="B13" s="50">
+        <v>45756</v>
+      </c>
       <c r="C13" s="51"/>
-      <c r="D13" s="52"/>
-      <c r="E13" s="53"/>
-      <c r="F13" s="36"/>
+      <c r="D13" s="52">
+        <v>50</v>
+      </c>
+      <c r="E13" s="53" t="s">
+        <v>4</v>
+      </c>
+      <c r="F13" s="36" t="s">
+        <v>36</v>
+      </c>
       <c r="G13" s="56"/>
       <c r="M13" t="s">
         <v>8</v>
@@ -2281,15 +2317,23 @@
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A14" s="8" t="str">
+      <c r="A14" s="8">
         <f>IF(ISBLANK(B14),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B14))</f>
-        <v/>
-      </c>
-      <c r="B14" s="46"/>
+        <v>15</v>
+      </c>
+      <c r="B14" s="46">
+        <v>45756</v>
+      </c>
       <c r="C14" s="47"/>
-      <c r="D14" s="48"/>
-      <c r="E14" s="49"/>
-      <c r="F14" s="36"/>
+      <c r="D14" s="48">
+        <v>5</v>
+      </c>
+      <c r="E14" s="49" t="s">
+        <v>22</v>
+      </c>
+      <c r="F14" s="36" t="s">
+        <v>37</v>
+      </c>
       <c r="G14" s="55"/>
       <c r="M14" t="s">
         <v>21</v>
@@ -2302,14 +2346,20 @@
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A15" s="16" t="str">
+      <c r="A15" s="16">
         <f>IF(ISBLANK(B15),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B15))</f>
-        <v/>
-      </c>
-      <c r="B15" s="50"/>
+        <v>15</v>
+      </c>
+      <c r="B15" s="50">
+        <v>45756</v>
+      </c>
       <c r="C15" s="51"/>
-      <c r="D15" s="52"/>
-      <c r="E15" s="53"/>
+      <c r="D15" s="52">
+        <v>5</v>
+      </c>
+      <c r="E15" s="53" t="s">
+        <v>22</v>
+      </c>
       <c r="F15" s="36"/>
       <c r="G15" s="56"/>
       <c r="M15" t="s">
@@ -2323,14 +2373,20 @@
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A16" s="8" t="str">
+      <c r="A16" s="8">
         <f>IF(ISBLANK(B16),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B16))</f>
-        <v/>
-      </c>
-      <c r="B16" s="46"/>
+        <v>15</v>
+      </c>
+      <c r="B16" s="46">
+        <v>45756</v>
+      </c>
       <c r="C16" s="47"/>
-      <c r="D16" s="48"/>
-      <c r="E16" s="49"/>
+      <c r="D16" s="48">
+        <v>5</v>
+      </c>
+      <c r="E16" s="49" t="s">
+        <v>22</v>
+      </c>
       <c r="F16" s="36"/>
       <c r="G16" s="55"/>
       <c r="O16">
@@ -8639,7 +8695,7 @@
       </c>
       <c r="B5">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Analyse!C5,'Journal de travail'!$D$7:$D$532)</f>
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="C5" s="41" t="str">
         <f>'Journal de travail'!M9</f>
@@ -8647,7 +8703,7 @@
       </c>
       <c r="D5" s="33">
         <f t="shared" ref="D5:D11" si="0">(A5+B5)/1440</f>
-        <v>0</v>
+        <v>3.4722222222222224E-2</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
@@ -8729,7 +8785,7 @@
       </c>
       <c r="B10">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Analyse!C10,'Journal de travail'!$D$7:$D$532)</f>
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="C10" s="37" t="str">
         <f>'Journal de travail'!M14</f>
@@ -8737,7 +8793,7 @@
       </c>
       <c r="D10" s="33">
         <f t="shared" si="0"/>
-        <v>1.3888888888888888E-2</v>
+        <v>3.4722222222222224E-2</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
@@ -8747,7 +8803,7 @@
       </c>
       <c r="B11">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Analyse!C11,'Journal de travail'!$D$7:$D$532)</f>
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="C11" s="39" t="str">
         <f>'Journal de travail'!M15</f>
@@ -8755,7 +8811,7 @@
       </c>
       <c r="D11" s="33">
         <f t="shared" si="0"/>
-        <v>1.3888888888888888E-2</v>
+        <v>2.4305555555555556E-2</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
@@ -8764,7 +8820,7 @@
       </c>
       <c r="D12" s="34">
         <f>SUM(D4:D11)</f>
-        <v>6.25E-2</v>
+        <v>0.12847222222222224</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
@@ -9001,6 +9057,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="be0d3259-a7ce-4623-88ec-81594dfcbc1c" xsi:nil="true"/>
@@ -9009,15 +9074,6 @@
     </lcf76f155ced4ddcb4097134ff3c332f>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -9040,6 +9096,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -9048,12 +9112,4 @@
     <ds:schemaRef ds:uri="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
dossier preuve vidéo, avec une vidéo représentative, qui preuve le bon marche d'application
</commit_message>
<xml_diff>
--- a/documentation/JDT-personal/Journal-de-Travail_NademoYosef.xlsx
+++ b/documentation/JDT-personal/Journal-de-Travail_NademoYosef.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pn25kdv\Documents\GitHub\Passion_lecture_FRONTEND\documentation\JDT-personal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15179ACD-243B-4EFE-A21E-4605C6F42EC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C820ED38-6FAC-4BD9-936A-FDDA363125EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="Mvap2W10CJFFJsnvkGXSiMLvpngxTMJbJsIKFe7Hzjn0XDcmjGuvBC2FjUCZ/hpRpUhUrG1T4kBlDAIo3yqmSQ==" workbookSaltValue="KXjgXOcsUZI/j7UgPKltzw==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="39">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -155,6 +155,9 @@
   </si>
   <si>
     <t>dossier routes, avec une liste des routes, photo de liste des routes, et tableau des routes</t>
+  </si>
+  <si>
+    <t>dossier preuve vidéo, avec une vidéo représentative, qui preuve le bon marche d'application</t>
   </si>
 </sst>
 </file>
@@ -2360,7 +2363,9 @@
       <c r="E15" s="53" t="s">
         <v>22</v>
       </c>
-      <c r="F15" s="36"/>
+      <c r="F15" s="36" t="s">
+        <v>38</v>
+      </c>
       <c r="G15" s="56"/>
       <c r="M15" t="s">
         <v>22</v>
@@ -9057,15 +9062,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="be0d3259-a7ce-4623-88ec-81594dfcbc1c" xsi:nil="true"/>
@@ -9074,6 +9070,15 @@
     </lcf76f155ced4ddcb4097134ff3c332f>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -9096,14 +9101,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -9112,4 +9109,12 @@
     <ds:schemaRef ds:uri="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
dossier DB(shemas), avec photos 2 représentation schématique du fonctionnement de la base de données (MCD et MLD), avec code pour créer la base de données, le programme Sider et Looping, dans lequel se trouvent des modèles (MLD et MCD).
dossier DB(shemas), avec photos 2 représentation schématique du fonctionnement de la base de données (MCD et MLD), avec code pour créer la base de données, le programme Sider et Looping, dans lequel se trouvent des modèles (MLD et MCD). jdt
</commit_message>
<xml_diff>
--- a/documentation/JDT-personal/Journal-de-Travail_NademoYosef.xlsx
+++ b/documentation/JDT-personal/Journal-de-Travail_NademoYosef.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pn25kdv\Documents\GitHub\Passion_lecture_FRONTEND\documentation\JDT-personal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C820ED38-6FAC-4BD9-936A-FDDA363125EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C87A4904-FA72-4ADF-AC71-0C68C368F03B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="Mvap2W10CJFFJsnvkGXSiMLvpngxTMJbJsIKFe7Hzjn0XDcmjGuvBC2FjUCZ/hpRpUhUrG1T4kBlDAIo3yqmSQ==" workbookSaltValue="KXjgXOcsUZI/j7UgPKltzw==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="41">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -158,6 +158,12 @@
   </si>
   <si>
     <t>dossier preuve vidéo, avec une vidéo représentative, qui preuve le bon marche d'application</t>
+  </si>
+  <si>
+    <t>dossier DB(shemas), avec photos 2 représentation schématique du fonctionnement de la base de données (MCD et MLD), avec code pour créer la base de données, le programme Sider et Looping, dans lequel se trouvent des modèles (MLD et MCD).</t>
+  </si>
+  <si>
+    <t>IN PROGRESS 🚧⏳🔄🔜</t>
   </si>
 </sst>
 </file>
@@ -2250,7 +2256,9 @@
       <c r="F11" s="36" t="s">
         <v>35</v>
       </c>
-      <c r="G11" s="56"/>
+      <c r="G11" s="56" t="s">
+        <v>40</v>
+      </c>
       <c r="M11" t="s">
         <v>6</v>
       </c>
@@ -2279,7 +2287,9 @@
       <c r="F12" s="36" t="s">
         <v>34</v>
       </c>
-      <c r="G12" s="55"/>
+      <c r="G12" s="55" t="s">
+        <v>40</v>
+      </c>
       <c r="M12" t="s">
         <v>7</v>
       </c>
@@ -2308,7 +2318,9 @@
       <c r="F13" s="36" t="s">
         <v>36</v>
       </c>
-      <c r="G13" s="56"/>
+      <c r="G13" s="56" t="s">
+        <v>40</v>
+      </c>
       <c r="M13" t="s">
         <v>8</v>
       </c>
@@ -2377,7 +2389,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:15" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A16" s="8">
         <f>IF(ISBLANK(B16),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B16))</f>
         <v>15</v>
@@ -2392,7 +2404,9 @@
       <c r="E16" s="49" t="s">
         <v>22</v>
       </c>
-      <c r="F16" s="36"/>
+      <c r="F16" s="36" t="s">
+        <v>39</v>
+      </c>
       <c r="G16" s="55"/>
       <c r="O16">
         <v>40</v>

</xml_diff>

<commit_message>
dossier Insomnia, Structure Insomnia
dossier Insomnia, Structure Insomnia: création des dossiers par type de route et ajout des requêtes HTTP pour chaque endpoint. Organise les requêtes Insomnia : création de dossiers pour chaque groupe de routes (auth, categories, books, etc.) avec les méthodes HTTP correspondantes
</commit_message>
<xml_diff>
--- a/documentation/JDT-personal/Journal-de-Travail_NademoYosef.xlsx
+++ b/documentation/JDT-personal/Journal-de-Travail_NademoYosef.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pn25kdv\Documents\GitHub\Passion_lecture_FRONTEND\documentation\JDT-personal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C87A4904-FA72-4ADF-AC71-0C68C368F03B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8583610-6C01-4017-A180-99C134C67888}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="Mvap2W10CJFFJsnvkGXSiMLvpngxTMJbJsIKFe7Hzjn0XDcmjGuvBC2FjUCZ/hpRpUhUrG1T4kBlDAIo3yqmSQ==" workbookSaltValue="KXjgXOcsUZI/j7UgPKltzw==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="43">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -164,6 +164,12 @@
   </si>
   <si>
     <t>IN PROGRESS 🚧⏳🔄🔜</t>
+  </si>
+  <si>
+    <t>dossier Insomnia, Structure Insomnia: création des dossiers par type de route et ajout des requêtes HTTP pour chaque endpoint. Organise les requêtes Insomnia : création de dossiers pour chaque groupe de routes (auth, categories, books, etc.) avec les méthodes HTTP correspondantes</t>
+  </si>
+  <si>
+    <t>✅</t>
   </si>
 </sst>
 </file>
@@ -1112,7 +1118,7 @@
                   <c:v>3.4722222222222224E-2</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>2.4305555555555556E-2</c:v>
+                  <c:v>2.7777777777777776E-2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2072,7 +2078,7 @@
       </c>
       <c r="C3" s="22" t="str">
         <f>INT(E4/1440)&amp;" jours "&amp;INT(MOD(E4/1440,1)*24)&amp;" heurs "&amp;INT(MOD(MOD(E4/1440,1)*24,1)*60)&amp;" minutes"</f>
-        <v>0 jours 3 heurs 4 minutes</v>
+        <v>0 jours 3 heurs 10 minutes</v>
       </c>
       <c r="D3" s="22"/>
       <c r="E3" s="3"/>
@@ -2091,11 +2097,11 @@
       </c>
       <c r="D4" s="22">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="E4" s="40">
         <f>SUM(C4:D4)</f>
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="7"/>
@@ -2349,7 +2355,9 @@
       <c r="F14" s="36" t="s">
         <v>37</v>
       </c>
-      <c r="G14" s="55"/>
+      <c r="G14" s="55" t="s">
+        <v>42</v>
+      </c>
       <c r="M14" t="s">
         <v>21</v>
       </c>
@@ -2378,7 +2386,9 @@
       <c r="F15" s="36" t="s">
         <v>38</v>
       </c>
-      <c r="G15" s="56"/>
+      <c r="G15" s="56" t="s">
+        <v>42</v>
+      </c>
       <c r="M15" t="s">
         <v>22</v>
       </c>
@@ -2407,22 +2417,34 @@
       <c r="F16" s="36" t="s">
         <v>39</v>
       </c>
-      <c r="G16" s="55"/>
+      <c r="G16" s="55" t="s">
+        <v>42</v>
+      </c>
       <c r="O16">
         <v>40</v>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A17" s="16" t="str">
+    <row r="17" spans="1:15" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="A17" s="16">
         <f>IF(ISBLANK(B17),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B17))</f>
-        <v/>
-      </c>
-      <c r="B17" s="50"/>
+        <v>15</v>
+      </c>
+      <c r="B17" s="50">
+        <v>45756</v>
+      </c>
       <c r="C17" s="51"/>
-      <c r="D17" s="52"/>
-      <c r="E17" s="53"/>
-      <c r="F17" s="36"/>
-      <c r="G17" s="56"/>
+      <c r="D17" s="52">
+        <v>5</v>
+      </c>
+      <c r="E17" s="53" t="s">
+        <v>22</v>
+      </c>
+      <c r="F17" s="36" t="s">
+        <v>41</v>
+      </c>
+      <c r="G17" s="56" t="s">
+        <v>42</v>
+      </c>
       <c r="O17">
         <v>45</v>
       </c>
@@ -8822,7 +8844,7 @@
       </c>
       <c r="B11">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Analyse!C11,'Journal de travail'!$D$7:$D$532)</f>
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="C11" s="39" t="str">
         <f>'Journal de travail'!M15</f>
@@ -8830,7 +8852,7 @@
       </c>
       <c r="D11" s="33">
         <f t="shared" si="0"/>
-        <v>2.4305555555555556E-2</v>
+        <v>2.7777777777777776E-2</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
@@ -8839,7 +8861,7 @@
       </c>
       <c r="D12" s="34">
         <f>SUM(D4:D11)</f>
-        <v>0.12847222222222224</v>
+        <v>0.13194444444444445</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
@@ -9076,6 +9098,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="be0d3259-a7ce-4623-88ec-81594dfcbc1c" xsi:nil="true"/>
@@ -9084,15 +9115,6 @@
     </lcf76f155ced4ddcb4097134ff3c332f>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -9115,6 +9137,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -9123,12 +9153,4 @@
     <ds:schemaRef ds:uri="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
construction du docker(création des fichiers .env, .yml, .dockerfile pour avoir l'environnement nécessaire au développement de l'application web.), container application,migration
# MySQL Database Configuration ENV     #sequelize  #.yml #.dockerfile #app.js
</commit_message>
<xml_diff>
--- a/documentation/JDT-personal/Journal-de-Travail_NademoYosef.xlsx
+++ b/documentation/JDT-personal/Journal-de-Travail_NademoYosef.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pn25kdv\Documents\GitHub\Passion_lecture_FRONTEND\documentation\JDT-personal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0EA7952-C53C-41D1-840A-57D3CCD55886}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82E00B7A-451E-43B3-B73E-1070ED7B4D09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="Mvap2W10CJFFJsnvkGXSiMLvpngxTMJbJsIKFe7Hzjn0XDcmjGuvBC2FjUCZ/hpRpUhUrG1T4kBlDAIo3yqmSQ==" workbookSaltValue="KXjgXOcsUZI/j7UgPKltzw==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
@@ -151,9 +151,6 @@
     <t>création du design de la page d'accueil</t>
   </si>
   <si>
-    <t>construction du docker(création des fichiers .env, .yml, .dockerfile pour avoir l'environnement nécessaire au développement de l'application web.)</t>
-  </si>
-  <si>
     <t>dossier routes, avec une liste des routes, photo de liste des routes, et tableau des routes</t>
   </si>
   <si>
@@ -163,9 +160,6 @@
     <t>dossier DB(shemas), avec photos 2 représentation schématique du fonctionnement de la base de données (MCD et MLD), avec code pour créer la base de données, le programme Sider et Looping, dans lequel se trouvent des modèles (MLD et MCD).</t>
   </si>
   <si>
-    <t>IN PROGRESS 🚧⏳🔄🔜</t>
-  </si>
-  <si>
     <t>dossier Insomnia, Structure Insomnia: création des dossiers par type de route et ajout des requêtes HTTP pour chaque endpoint. Organise les requêtes Insomnia : création de dossiers pour chaque groupe de routes (auth, categories, books, etc.) avec les méthodes HTTP correspondantes</t>
   </si>
   <si>
@@ -173,6 +167,12 @@
   </si>
   <si>
     <t>Ajout du dossier 'code' avec la structure complète du projet : package.json, fichiers .yml, .env, etc. (code complet du projet 295)</t>
+  </si>
+  <si>
+    <t>construction du docker(création des fichiers .env, .yml, .dockerfile pour avoir l'environnement nécessaire au développement de l'application web.), container application,migration</t>
+  </si>
+  <si>
+    <t># MySQL Database Configuration ENV; # MySQL Database Configuration ENV     #sequelize  #.yml #.dockerfile #app.js      Command:         docker-compose --env-file .env up --build</t>
   </si>
 </sst>
 </file>
@@ -2309,7 +2309,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="1:15" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A13" s="16">
         <f>IF(ISBLANK(B13),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B13))</f>
         <v>15</v>
@@ -2325,10 +2325,10 @@
         <v>4</v>
       </c>
       <c r="F13" s="36" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="G13" s="56" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="M13" t="s">
         <v>8</v>
@@ -2356,10 +2356,10 @@
         <v>22</v>
       </c>
       <c r="F14" s="36" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G14" s="55" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="M14" t="s">
         <v>21</v>
@@ -2387,10 +2387,10 @@
         <v>22</v>
       </c>
       <c r="F15" s="36" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="G15" s="56" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="M15" t="s">
         <v>22</v>
@@ -2418,10 +2418,10 @@
         <v>22</v>
       </c>
       <c r="F16" s="36" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G16" s="55" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="O16">
         <v>40</v>
@@ -2443,10 +2443,10 @@
         <v>22</v>
       </c>
       <c r="F17" s="36" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="G17" s="56" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="O17">
         <v>45</v>
@@ -2468,10 +2468,10 @@
         <v>22</v>
       </c>
       <c r="F18" s="36" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="G18" s="55" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="O18">
         <v>50</v>
@@ -9111,6 +9111,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="be0d3259-a7ce-4623-88ec-81594dfcbc1c" xsi:nil="true"/>
@@ -9119,15 +9128,6 @@
     </lcf76f155ced4ddcb4097134ff3c332f>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -9150,6 +9150,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -9158,12 +9166,4 @@
     <ds:schemaRef ds:uri="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Chore(Journal De travail Yosef)
[DONE] [20min]
- Update journal de travail
</commit_message>
<xml_diff>
--- a/documentation/JDT-personal/Journal-de-Travail_NademoYosef.xlsx
+++ b/documentation/JDT-personal/Journal-de-Travail_NademoYosef.xlsx
@@ -8,10 +8,10 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pn25kdv\Documents\GitHub\Passion_lecture_FRONTEND\documentation\JDT-personal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82E00B7A-451E-43B3-B73E-1070ED7B4D09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{192CEB1C-8981-43BA-85ED-3AFF7EC25057}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="Mvap2W10CJFFJsnvkGXSiMLvpngxTMJbJsIKFe7Hzjn0XDcmjGuvBC2FjUCZ/hpRpUhUrG1T4kBlDAIo3yqmSQ==" workbookSaltValue="KXjgXOcsUZI/j7UgPKltzw==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
+    <workbookView xWindow="4830" yWindow="0" windowWidth="21600" windowHeight="15600" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal de travail" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="48">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -173,6 +173,18 @@
   </si>
   <si>
     <t># MySQL Database Configuration ENV; # MySQL Database Configuration ENV     #sequelize  #.yml #.dockerfile #app.js      Command:         docker-compose --env-file .env up --build</t>
+  </si>
+  <si>
+    <t>création du design de la page d’ajout d’un ouvrage (accès utilisateur) 1ere version</t>
+  </si>
+  <si>
+    <t>devloppement du footer, en utilisant le design Figma</t>
+  </si>
+  <si>
+    <t>devloppement du de la page d'accueil, en utilisant le design Figma</t>
+  </si>
+  <si>
+    <t>J’ai mis à jour mon journal de travail en notant les tâches effectuées, les points à améliorer et les prochaines étapes à suivre.</t>
   </si>
 </sst>
 </file>
@@ -1103,13 +1115,13 @@
                   <c:v>1.3888888888888888E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>3.4722222222222224E-2</c:v>
+                  <c:v>0.11805555555555555</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>1.3888888888888888E-2</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>2.0833333333333332E-2</c:v>
@@ -1118,7 +1130,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>3.4722222222222224E-2</c:v>
+                  <c:v>4.8611111111111112E-2</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>3.125E-2</c:v>
@@ -2081,7 +2093,7 @@
       </c>
       <c r="C3" s="22" t="str">
         <f>INT(E4/1440)&amp;" jours "&amp;INT(MOD(E4/1440,1)*24)&amp;" heurs "&amp;INT(MOD(MOD(E4/1440,1)*24,1)*60)&amp;" minutes"</f>
-        <v>0 jours 3 heurs 15 minutes</v>
+        <v>0 jours 5 heurs 55 minutes</v>
       </c>
       <c r="D3" s="22"/>
       <c r="E3" s="3"/>
@@ -2096,15 +2108,15 @@
       <c r="B4" s="5"/>
       <c r="C4" s="22">
         <f>SUBTOTAL(9,$C$7:$C$531)*60</f>
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="D4" s="22">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>195</v>
+        <v>295</v>
       </c>
       <c r="E4" s="40">
         <f>SUM(C4:D4)</f>
-        <v>195</v>
+        <v>355</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="7"/>
@@ -2236,7 +2248,9 @@
       <c r="F10" s="36" t="s">
         <v>33</v>
       </c>
-      <c r="G10" s="55"/>
+      <c r="G10" s="55" t="s">
+        <v>40</v>
+      </c>
       <c r="M10" t="s">
         <v>5</v>
       </c>
@@ -2478,54 +2492,88 @@
       </c>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A19" s="16" t="str">
+      <c r="A19" s="16">
         <f>IF(ISBLANK(B19),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B19))</f>
-        <v/>
-      </c>
-      <c r="B19" s="50"/>
+        <v>18</v>
+      </c>
+      <c r="B19" s="50">
+        <v>45777</v>
+      </c>
       <c r="C19" s="51"/>
-      <c r="D19" s="52"/>
-      <c r="E19" s="53"/>
-      <c r="F19" s="36"/>
+      <c r="D19" s="52">
+        <v>20</v>
+      </c>
+      <c r="E19" s="53" t="s">
+        <v>21</v>
+      </c>
+      <c r="F19" s="36" t="s">
+        <v>44</v>
+      </c>
       <c r="G19" s="56"/>
       <c r="O19">
         <v>55</v>
       </c>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A20" s="8" t="str">
+      <c r="A20" s="8">
         <f>IF(ISBLANK(B20),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B20))</f>
-        <v/>
-      </c>
-      <c r="B20" s="46"/>
+        <v>18</v>
+      </c>
+      <c r="B20" s="46">
+        <v>45777</v>
+      </c>
       <c r="C20" s="47"/>
-      <c r="D20" s="48"/>
-      <c r="E20" s="49"/>
-      <c r="F20" s="36"/>
+      <c r="D20" s="48">
+        <v>30</v>
+      </c>
+      <c r="E20" s="49" t="s">
+        <v>4</v>
+      </c>
+      <c r="F20" s="36" t="s">
+        <v>45</v>
+      </c>
       <c r="G20" s="55"/>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A21" s="16" t="str">
+      <c r="A21" s="16">
         <f>IF(ISBLANK(B21),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B21))</f>
-        <v/>
-      </c>
-      <c r="B21" s="50"/>
-      <c r="C21" s="51"/>
-      <c r="D21" s="52"/>
-      <c r="E21" s="53"/>
-      <c r="F21" s="36"/>
+        <v>18</v>
+      </c>
+      <c r="B21" s="50">
+        <v>45777</v>
+      </c>
+      <c r="C21" s="51">
+        <v>1</v>
+      </c>
+      <c r="D21" s="52">
+        <v>30</v>
+      </c>
+      <c r="E21" s="53" t="s">
+        <v>4</v>
+      </c>
+      <c r="F21" s="36" t="s">
+        <v>46</v>
+      </c>
       <c r="G21" s="56"/>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A22" s="8" t="str">
+    <row r="22" spans="1:15" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A22" s="8">
         <f>IF(ISBLANK(B22),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B22))</f>
-        <v/>
-      </c>
-      <c r="B22" s="46"/>
+        <v>18</v>
+      </c>
+      <c r="B22" s="46">
+        <v>45777</v>
+      </c>
       <c r="C22" s="47"/>
-      <c r="D22" s="48"/>
-      <c r="E22" s="49"/>
-      <c r="F22" s="36"/>
+      <c r="D22" s="48">
+        <v>20</v>
+      </c>
+      <c r="E22" s="49" t="s">
+        <v>6</v>
+      </c>
+      <c r="F22" s="36" t="s">
+        <v>47</v>
+      </c>
       <c r="G22" s="55"/>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.25">
@@ -8745,11 +8793,11 @@
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Analyse!C5,'Journal de travail'!$C$7:$C$532)*60</f>
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="B5">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Analyse!C5,'Journal de travail'!$D$7:$D$532)</f>
-        <v>50</v>
+        <v>110</v>
       </c>
       <c r="C5" s="41" t="str">
         <f>'Journal de travail'!M9</f>
@@ -8757,7 +8805,7 @@
       </c>
       <c r="D5" s="33">
         <f t="shared" ref="D5:D11" si="0">(A5+B5)/1440</f>
-        <v>3.4722222222222224E-2</v>
+        <v>0.11805555555555555</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
@@ -8785,7 +8833,7 @@
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Analyse!C7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="C7" s="27" t="str">
         <f>'Journal de travail'!M11</f>
@@ -8793,7 +8841,7 @@
       </c>
       <c r="D7" s="33">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1.3888888888888888E-2</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
@@ -8839,7 +8887,7 @@
       </c>
       <c r="B10">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Analyse!C10,'Journal de travail'!$D$7:$D$532)</f>
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="C10" s="37" t="str">
         <f>'Journal de travail'!M14</f>
@@ -8847,7 +8895,7 @@
       </c>
       <c r="D10" s="33">
         <f t="shared" si="0"/>
-        <v>3.4722222222222224E-2</v>
+        <v>4.8611111111111112E-2</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
@@ -8874,7 +8922,7 @@
       </c>
       <c r="D12" s="34">
         <f>SUM(D4:D11)</f>
-        <v>0.13541666666666669</v>
+        <v>0.24652777777777779</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
@@ -8888,6 +8936,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D4F20F00DBE2EE49BE9523363A2DF18B" ma:contentTypeVersion="13" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="313dbdbec26224d1c2bb7e3c488b2a4e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="99ffe1f3-7857-457f-add0-5bdef636f38d" xmlns:ns3="be0d3259-a7ce-4623-88ec-81594dfcbc1c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4739345e3d2c6be79c5ae1a54d02a4a7" ns2:_="" ns3:_="">
     <xsd:import namespace="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
@@ -9110,15 +9167,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -9131,6 +9179,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F2FB702A-DCBD-43A8-A34C-6000FD8861AD}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -9149,14 +9205,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
DESIGN - Figma(Une page d’ajout d’un ouvrage)
[DONE] [20min]
- Modélisation de maquette (Une page d’ajout d’un ouvrage)
</commit_message>
<xml_diff>
--- a/documentation/JDT-personal/Journal-de-Travail_NademoYosef.xlsx
+++ b/documentation/JDT-personal/Journal-de-Travail_NademoYosef.xlsx
@@ -8,10 +8,10 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pn25kdv\Documents\GitHub\Passion_lecture_FRONTEND\documentation\JDT-personal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{192CEB1C-8981-43BA-85ED-3AFF7EC25057}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC16B887-5448-4DED-A93C-5E2E79064CBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="Mvap2W10CJFFJsnvkGXSiMLvpngxTMJbJsIKFe7Hzjn0XDcmjGuvBC2FjUCZ/hpRpUhUrG1T4kBlDAIo3yqmSQ==" workbookSaltValue="KXjgXOcsUZI/j7UgPKltzw==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="4830" yWindow="0" windowWidth="21600" windowHeight="15600" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
+    <workbookView xWindow="4830" yWindow="960" windowWidth="21600" windowHeight="11385" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal de travail" sheetId="1" r:id="rId1"/>
@@ -8945,6 +8945,17 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="be0d3259-a7ce-4623-88ec-81594dfcbc1c" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="99ffe1f3-7857-457f-add0-5bdef636f38d">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D4F20F00DBE2EE49BE9523363A2DF18B" ma:contentTypeVersion="13" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="313dbdbec26224d1c2bb7e3c488b2a4e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="99ffe1f3-7857-457f-add0-5bdef636f38d" xmlns:ns3="be0d3259-a7ce-4623-88ec-81594dfcbc1c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4739345e3d2c6be79c5ae1a54d02a4a7" ns2:_="" ns3:_="">
     <xsd:import namespace="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
@@ -9167,17 +9178,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="be0d3259-a7ce-4623-88ec-81594dfcbc1c" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="99ffe1f3-7857-457f-add0-5bdef636f38d">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>
@@ -9187,6 +9187,17 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="be0d3259-a7ce-4623-88ec-81594dfcbc1c"/>
+    <ds:schemaRef ds:uri="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F2FB702A-DCBD-43A8-A34C-6000FD8861AD}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -9203,15 +9214,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="be0d3259-a7ce-4623-88ec-81594dfcbc1c"/>
-    <ds:schemaRef ds:uri="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Chore(Journal De travail Yosef
[DONE] [5min]
- Update journal de travail
</commit_message>
<xml_diff>
--- a/documentation/JDT-personal/Journal-de-Travail_NademoYosef.xlsx
+++ b/documentation/JDT-personal/Journal-de-Travail_NademoYosef.xlsx
@@ -8,10 +8,10 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pn25kdv\Documents\GitHub\Passion_lecture_FRONTEND\documentation\JDT-personal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC16B887-5448-4DED-A93C-5E2E79064CBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F06ED715-14FF-4610-AE75-431302D434B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="Mvap2W10CJFFJsnvkGXSiMLvpngxTMJbJsIKFe7Hzjn0XDcmjGuvBC2FjUCZ/hpRpUhUrG1T4kBlDAIo3yqmSQ==" workbookSaltValue="KXjgXOcsUZI/j7UgPKltzw==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="4830" yWindow="960" windowWidth="21600" windowHeight="11385" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
+    <workbookView xWindow="3210" yWindow="960" windowWidth="24840" windowHeight="12270" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal de travail" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="53">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -185,6 +185,21 @@
   </si>
   <si>
     <t>J’ai mis à jour mon journal de travail en notant les tâches effectuées, les points à améliorer et les prochaines étapes à suivre.</t>
+  </si>
+  <si>
+    <t>devloppement de App.vue</t>
+  </si>
+  <si>
+    <t>structurisation de App.vue , correction des erreurs ,creation des import export correctes - CSS  (Error message styling, buttons)</t>
+  </si>
+  <si>
+    <t>modification pour la  version anglaise</t>
+  </si>
+  <si>
+    <t>modification pour un champs ajout du champ "writer"</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> export du fichier maquette complet (un fichier pour réstorer la maquette)</t>
   </si>
 </sst>
 </file>
@@ -368,7 +383,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -504,11 +519,99 @@
     <xf numFmtId="20" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="17">
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0070C0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF7030A0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B0F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFCCCC00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -678,80 +781,6 @@
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
           <bgColor theme="2" tint="-9.9978637043366805E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF0070C0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="2" tint="-0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF7030A0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B0F0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFCCCC00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="-0.24994659260841701"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1115,7 +1144,7 @@
                   <c:v>1.3888888888888888E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.11805555555555555</c:v>
+                  <c:v>0.13194444444444445</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -1130,7 +1159,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>4.8611111111111112E-2</c:v>
+                  <c:v>5.5555555555555552E-2</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>3.125E-2</c:v>
@@ -1839,18 +1868,18 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F2213DF1-F6B1-174C-AC17-4E96BE96C00D}" name="Table1" displayName="Table1" ref="A6:G532" totalsRowShown="0" headerRowDxfId="8" tableBorderDxfId="7">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F2213DF1-F6B1-174C-AC17-4E96BE96C00D}" name="Table1" displayName="Table1" ref="A6:G532" totalsRowShown="0" headerRowDxfId="16" tableBorderDxfId="15">
   <autoFilter ref="A6:G532" xr:uid="{F2213DF1-F6B1-174C-AC17-4E96BE96C00D}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{315BA4B4-9BD9-AB4E-8D40-FABFA0BB2AEA}" name="Semaine" dataDxfId="6">
+    <tableColumn id="1" xr3:uid="{315BA4B4-9BD9-AB4E-8D40-FABFA0BB2AEA}" name="Semaine" dataDxfId="14">
       <calculatedColumnFormula>IF(ISBLANK(B7),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B7))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{503C31E9-854D-BF42-85AC-8DFA1376C4D8}" name="Jour" dataDxfId="5"/>
-    <tableColumn id="3" xr3:uid="{B35A0B98-71A0-BA4F-BFAB-00A05EA1F23A}" name="heure" dataDxfId="4"/>
-    <tableColumn id="4" xr3:uid="{BE4D837D-FC99-BA48-A82F-B8C8E4CE5BF8}" name="min." dataDxfId="3"/>
-    <tableColumn id="5" xr3:uid="{A2DCC539-6D2A-B04A-BF8E-6FACE6268D1F}" name="Activité" dataDxfId="2"/>
-    <tableColumn id="6" xr3:uid="{4EA406B9-7EF7-D547-AF98-5AD11BE168E9}" name="Description" dataDxfId="1"/>
-    <tableColumn id="7" xr3:uid="{1735360B-2647-6D42-A0E3-3425EE302FFD}" name="Remarque / problème" dataDxfId="0"/>
+    <tableColumn id="2" xr3:uid="{503C31E9-854D-BF42-85AC-8DFA1376C4D8}" name="Jour" dataDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{B35A0B98-71A0-BA4F-BFAB-00A05EA1F23A}" name="heure" dataDxfId="12"/>
+    <tableColumn id="4" xr3:uid="{BE4D837D-FC99-BA48-A82F-B8C8E4CE5BF8}" name="min." dataDxfId="11"/>
+    <tableColumn id="5" xr3:uid="{A2DCC539-6D2A-B04A-BF8E-6FACE6268D1F}" name="Activité" dataDxfId="10"/>
+    <tableColumn id="6" xr3:uid="{4EA406B9-7EF7-D547-AF98-5AD11BE168E9}" name="Description" dataDxfId="9"/>
+    <tableColumn id="7" xr3:uid="{1735360B-2647-6D42-A0E3-3425EE302FFD}" name="Remarque / problème" dataDxfId="8"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2093,7 +2122,7 @@
       </c>
       <c r="C3" s="22" t="str">
         <f>INT(E4/1440)&amp;" jours "&amp;INT(MOD(E4/1440,1)*24)&amp;" heurs "&amp;INT(MOD(MOD(E4/1440,1)*24,1)*60)&amp;" minutes"</f>
-        <v>0 jours 5 heurs 55 minutes</v>
+        <v>0 jours 6 heurs 25 minutes</v>
       </c>
       <c r="D3" s="22"/>
       <c r="E3" s="3"/>
@@ -2112,11 +2141,11 @@
       </c>
       <c r="D4" s="22">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>295</v>
+        <v>325</v>
       </c>
       <c r="E4" s="40">
         <f>SUM(C4:D4)</f>
-        <v>355</v>
+        <v>385</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="7"/>
@@ -2534,7 +2563,7 @@
       </c>
       <c r="G20" s="55"/>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:15" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A21" s="16">
         <f>IF(ISBLANK(B21),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B21))</f>
         <v>18</v>
@@ -2542,21 +2571,21 @@
       <c r="B21" s="50">
         <v>45777</v>
       </c>
-      <c r="C21" s="51">
-        <v>1</v>
-      </c>
+      <c r="C21" s="51"/>
       <c r="D21" s="52">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="E21" s="53" t="s">
         <v>4</v>
       </c>
       <c r="F21" s="36" t="s">
-        <v>46</v>
-      </c>
-      <c r="G21" s="56"/>
-    </row>
-    <row r="22" spans="1:15" ht="31.5" x14ac:dyDescent="0.25">
+        <v>48</v>
+      </c>
+      <c r="G21" s="56" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" s="8">
         <f>IF(ISBLANK(B22),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B22))</f>
         <v>18</v>
@@ -2566,50 +2595,78 @@
       </c>
       <c r="C22" s="47"/>
       <c r="D22" s="48">
+        <v>5</v>
+      </c>
+      <c r="E22" s="49" t="s">
+        <v>21</v>
+      </c>
+      <c r="F22" s="36" t="s">
+        <v>50</v>
+      </c>
+      <c r="G22" s="55"/>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A23" s="16">
+        <f>IF(ISBLANK(B23),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B23))</f>
+        <v>18</v>
+      </c>
+      <c r="B23" s="50">
+        <v>45777</v>
+      </c>
+      <c r="C23" s="51"/>
+      <c r="D23" s="52">
+        <v>5</v>
+      </c>
+      <c r="E23" s="53" t="s">
+        <v>21</v>
+      </c>
+      <c r="F23" s="36" t="s">
+        <v>51</v>
+      </c>
+      <c r="G23" s="56" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A24" s="8">
+        <f>IF(ISBLANK(B24),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B24))</f>
+        <v>18</v>
+      </c>
+      <c r="B24" s="46">
+        <v>45777</v>
+      </c>
+      <c r="C24" s="47">
+        <v>1</v>
+      </c>
+      <c r="D24" s="48">
+        <v>30</v>
+      </c>
+      <c r="E24" s="49" t="s">
+        <v>4</v>
+      </c>
+      <c r="F24" s="36" t="s">
+        <v>46</v>
+      </c>
+      <c r="G24" s="55"/>
+    </row>
+    <row r="25" spans="1:15" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A25" s="16">
+        <f>IF(ISBLANK(B25),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B25))</f>
+        <v>18</v>
+      </c>
+      <c r="B25" s="50">
+        <v>45777</v>
+      </c>
+      <c r="C25" s="51"/>
+      <c r="D25" s="52">
         <v>20</v>
       </c>
-      <c r="E22" s="49" t="s">
+      <c r="E25" s="53" t="s">
         <v>6</v>
       </c>
-      <c r="F22" s="36" t="s">
+      <c r="F25" s="36" t="s">
         <v>47</v>
       </c>
-      <c r="G22" s="55"/>
-    </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A23" s="16" t="str">
-        <f>IF(ISBLANK(B23),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B23))</f>
-        <v/>
-      </c>
-      <c r="B23" s="50"/>
-      <c r="C23" s="51"/>
-      <c r="D23" s="52"/>
-      <c r="E23" s="53"/>
-      <c r="F23" s="36"/>
-      <c r="G23" s="56"/>
-    </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A24" s="8" t="str">
-        <f>IF(ISBLANK(B24),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B24))</f>
-        <v/>
-      </c>
-      <c r="B24" s="46"/>
-      <c r="C24" s="47"/>
-      <c r="D24" s="48"/>
-      <c r="E24" s="49"/>
-      <c r="F24" s="36"/>
-      <c r="G24" s="55"/>
-    </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A25" s="16" t="str">
-        <f>IF(ISBLANK(B25),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B25))</f>
-        <v/>
-      </c>
-      <c r="B25" s="50"/>
-      <c r="C25" s="51"/>
-      <c r="D25" s="52"/>
-      <c r="E25" s="53"/>
-      <c r="F25" s="36"/>
       <c r="G25" s="56"/>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.25">
@@ -2618,10 +2675,10 @@
         <v/>
       </c>
       <c r="B26" s="46"/>
-      <c r="C26" s="47"/>
-      <c r="D26" s="48"/>
-      <c r="E26" s="49"/>
-      <c r="F26" s="36"/>
+      <c r="C26" s="59"/>
+      <c r="D26" s="60"/>
+      <c r="E26" s="61"/>
+      <c r="F26" s="62"/>
       <c r="G26" s="55"/>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.25">
@@ -2630,10 +2687,10 @@
         <v/>
       </c>
       <c r="B27" s="50"/>
-      <c r="C27" s="51"/>
-      <c r="D27" s="52"/>
-      <c r="E27" s="53"/>
-      <c r="F27" s="36"/>
+      <c r="C27" s="59"/>
+      <c r="D27" s="60"/>
+      <c r="E27" s="61"/>
+      <c r="F27" s="62"/>
       <c r="G27" s="56"/>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.25">
@@ -8702,40 +8759,40 @@
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="C5:D5"/>
   </mergeCells>
-  <conditionalFormatting sqref="E7:E532">
-    <cfRule type="expression" dxfId="16" priority="1">
+  <conditionalFormatting sqref="E28:E532 E7:E25">
+    <cfRule type="expression" dxfId="7" priority="1">
       <formula>$E7="Autre"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="15" priority="2" stopIfTrue="1">
+    <cfRule type="expression" dxfId="6" priority="2" stopIfTrue="1">
       <formula>$E7="Design"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="14" priority="3" stopIfTrue="1">
+    <cfRule type="expression" dxfId="5" priority="3" stopIfTrue="1">
       <formula>$E7="Présentation"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="13" priority="4" stopIfTrue="1">
+    <cfRule type="expression" dxfId="4" priority="4" stopIfTrue="1">
       <formula>$E7="Meeting"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="12" priority="5" stopIfTrue="1">
+    <cfRule type="expression" dxfId="3" priority="5" stopIfTrue="1">
       <formula>$E7="Documentation"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="11" priority="6" stopIfTrue="1">
+    <cfRule type="expression" dxfId="2" priority="6" stopIfTrue="1">
       <formula>$E7="Test"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="10" priority="7" stopIfTrue="1">
+    <cfRule type="expression" dxfId="1" priority="7" stopIfTrue="1">
       <formula>$E7="Analyse"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="9" priority="9" stopIfTrue="1">
+    <cfRule type="expression" dxfId="0" priority="9" stopIfTrue="1">
       <formula>$E7="Développement"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C7:C532" xr:uid="{9D52E29F-610D-40B2-B3CC-F94A741DD978}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C28:C532 C7:C25" xr:uid="{9D52E29F-610D-40B2-B3CC-F94A741DD978}">
       <formula1>$N$7:$N$15</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D7:D532" xr:uid="{46510F84-8BCC-4BD6-9A19-9F03ACD74D05}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D28:D532 D7:D25" xr:uid="{46510F84-8BCC-4BD6-9A19-9F03ACD74D05}">
       <formula1>$O$7:$O$19</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E7:E532" xr:uid="{5717AF9A-5C26-4256-9473-8948342ED6D3}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E28:E532 E7:E25" xr:uid="{5717AF9A-5C26-4256-9473-8948342ED6D3}">
       <formula1>$M$7:$M$15</formula1>
     </dataValidation>
   </dataValidations>
@@ -8797,7 +8854,7 @@
       </c>
       <c r="B5">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Analyse!C5,'Journal de travail'!$D$7:$D$532)</f>
-        <v>110</v>
+        <v>130</v>
       </c>
       <c r="C5" s="41" t="str">
         <f>'Journal de travail'!M9</f>
@@ -8805,7 +8862,7 @@
       </c>
       <c r="D5" s="33">
         <f t="shared" ref="D5:D11" si="0">(A5+B5)/1440</f>
-        <v>0.11805555555555555</v>
+        <v>0.13194444444444445</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
@@ -8887,7 +8944,7 @@
       </c>
       <c r="B10">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Analyse!C10,'Journal de travail'!$D$7:$D$532)</f>
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="C10" s="37" t="str">
         <f>'Journal de travail'!M14</f>
@@ -8895,7 +8952,7 @@
       </c>
       <c r="D10" s="33">
         <f t="shared" si="0"/>
-        <v>4.8611111111111112E-2</v>
+        <v>5.5555555555555552E-2</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
@@ -8922,7 +8979,7 @@
       </c>
       <c r="D12" s="34">
         <f>SUM(D4:D11)</f>
-        <v>0.24652777777777779</v>
+        <v>0.26736111111111116</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
@@ -8945,17 +9002,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="be0d3259-a7ce-4623-88ec-81594dfcbc1c" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="99ffe1f3-7857-457f-add0-5bdef636f38d">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D4F20F00DBE2EE49BE9523363A2DF18B" ma:contentTypeVersion="13" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="313dbdbec26224d1c2bb7e3c488b2a4e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="99ffe1f3-7857-457f-add0-5bdef636f38d" xmlns:ns3="be0d3259-a7ce-4623-88ec-81594dfcbc1c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4739345e3d2c6be79c5ae1a54d02a4a7" ns2:_="" ns3:_="">
     <xsd:import namespace="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
@@ -9178,6 +9224,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="be0d3259-a7ce-4623-88ec-81594dfcbc1c" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="99ffe1f3-7857-457f-add0-5bdef636f38d">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>
@@ -9187,17 +9244,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="be0d3259-a7ce-4623-88ec-81594dfcbc1c"/>
-    <ds:schemaRef ds:uri="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F2FB702A-DCBD-43A8-A34C-6000FD8861AD}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -9214,4 +9260,15 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="be0d3259-a7ce-4623-88ec-81594dfcbc1c"/>
+    <ds:schemaRef ds:uri="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
BackEnd(supprimer un problème avec CORS)
BackEnd(supprimer un problème avec CORS), installation d paquet npm "cors", importation + autorise toutes les origines; TEST avec des images
</commit_message>
<xml_diff>
--- a/documentation/JDT-personal/Journal-de-Travail_NademoYosef.xlsx
+++ b/documentation/JDT-personal/Journal-de-Travail_NademoYosef.xlsx
@@ -8,10 +8,10 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pn25kdv\Documents\GitHub\Passion_lecture_FRONTEND\documentation\JDT-personal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F06ED715-14FF-4610-AE75-431302D434B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99DC3598-6B09-40B6-B3AD-952C1657E838}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="Mvap2W10CJFFJsnvkGXSiMLvpngxTMJbJsIKFe7Hzjn0XDcmjGuvBC2FjUCZ/hpRpUhUrG1T4kBlDAIo3yqmSQ==" workbookSaltValue="KXjgXOcsUZI/j7UgPKltzw==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="3210" yWindow="960" windowWidth="24840" windowHeight="12270" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
+    <workbookView xWindow="450" yWindow="1290" windowWidth="24840" windowHeight="12270" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal de travail" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="60">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -200,6 +200,27 @@
   </si>
   <si>
     <t xml:space="preserve"> export du fichier maquette complet (un fichier pour réstorer la maquette)</t>
+  </si>
+  <si>
+    <t>PageAcceuil(Book data loading from API, Books section (model))</t>
+  </si>
+  <si>
+    <t>20miv</t>
+  </si>
+  <si>
+    <t>BACKEND(app.js)</t>
+  </si>
+  <si>
+    <t>FRONTEND(Acceuil.vue)</t>
+  </si>
+  <si>
+    <t>donc j'ai mis l'information plus bas</t>
+  </si>
+  <si>
+    <t>ce champs est pas au norme(la partie "Activite")</t>
+  </si>
+  <si>
+    <t>BackEnd(supprimer un problème avec CORS), installation d paquet npm "cors", importation + autorise toutes les origines; TEST avec des images</t>
   </si>
 </sst>
 </file>
@@ -512,13 +533,6 @@
       <alignment wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="16" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
@@ -533,85 +547,18 @@
       <alignment wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="16" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="20" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="17">
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF0070C0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="2" tint="-0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF7030A0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B0F0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFCCCC00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -781,6 +728,80 @@
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
           <bgColor theme="2" tint="-9.9978637043366805E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0070C0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF7030A0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B0F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFCCCC00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="-0.24994659260841701"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1144,7 +1165,7 @@
                   <c:v>1.3888888888888888E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.13194444444444445</c:v>
+                  <c:v>0.15972222222222221</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -1868,18 +1889,18 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F2213DF1-F6B1-174C-AC17-4E96BE96C00D}" name="Table1" displayName="Table1" ref="A6:G532" totalsRowShown="0" headerRowDxfId="16" tableBorderDxfId="15">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F2213DF1-F6B1-174C-AC17-4E96BE96C00D}" name="Table1" displayName="Table1" ref="A6:G532" totalsRowShown="0" headerRowDxfId="8" tableBorderDxfId="7">
   <autoFilter ref="A6:G532" xr:uid="{F2213DF1-F6B1-174C-AC17-4E96BE96C00D}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{315BA4B4-9BD9-AB4E-8D40-FABFA0BB2AEA}" name="Semaine" dataDxfId="14">
+    <tableColumn id="1" xr3:uid="{315BA4B4-9BD9-AB4E-8D40-FABFA0BB2AEA}" name="Semaine" dataDxfId="6">
       <calculatedColumnFormula>IF(ISBLANK(B7),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B7))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{503C31E9-854D-BF42-85AC-8DFA1376C4D8}" name="Jour" dataDxfId="13"/>
-    <tableColumn id="3" xr3:uid="{B35A0B98-71A0-BA4F-BFAB-00A05EA1F23A}" name="heure" dataDxfId="12"/>
-    <tableColumn id="4" xr3:uid="{BE4D837D-FC99-BA48-A82F-B8C8E4CE5BF8}" name="min." dataDxfId="11"/>
-    <tableColumn id="5" xr3:uid="{A2DCC539-6D2A-B04A-BF8E-6FACE6268D1F}" name="Activité" dataDxfId="10"/>
-    <tableColumn id="6" xr3:uid="{4EA406B9-7EF7-D547-AF98-5AD11BE168E9}" name="Description" dataDxfId="9"/>
-    <tableColumn id="7" xr3:uid="{1735360B-2647-6D42-A0E3-3425EE302FFD}" name="Remarque / problème" dataDxfId="8"/>
+    <tableColumn id="2" xr3:uid="{503C31E9-854D-BF42-85AC-8DFA1376C4D8}" name="Jour" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{B35A0B98-71A0-BA4F-BFAB-00A05EA1F23A}" name="heure" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{BE4D837D-FC99-BA48-A82F-B8C8E4CE5BF8}" name="min." dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{A2DCC539-6D2A-B04A-BF8E-6FACE6268D1F}" name="Activité" dataDxfId="2"/>
+    <tableColumn id="6" xr3:uid="{4EA406B9-7EF7-D547-AF98-5AD11BE168E9}" name="Description" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{1735360B-2647-6D42-A0E3-3425EE302FFD}" name="Remarque / problème" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2104,11 +2125,11 @@
       <c r="B2" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="57" t="s">
+      <c r="C2" s="61" t="s">
         <v>27</v>
       </c>
-      <c r="D2" s="57"/>
-      <c r="E2" s="57"/>
+      <c r="D2" s="61"/>
+      <c r="E2" s="61"/>
       <c r="F2" s="5" t="s">
         <v>2</v>
       </c>
@@ -2122,7 +2143,7 @@
       </c>
       <c r="C3" s="22" t="str">
         <f>INT(E4/1440)&amp;" jours "&amp;INT(MOD(E4/1440,1)*24)&amp;" heurs "&amp;INT(MOD(MOD(E4/1440,1)*24,1)*60)&amp;" minutes"</f>
-        <v>0 jours 6 heurs 25 minutes</v>
+        <v>0 jours 7 heurs 5 minutes</v>
       </c>
       <c r="D3" s="22"/>
       <c r="E3" s="3"/>
@@ -2141,20 +2162,20 @@
       </c>
       <c r="D4" s="22">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>325</v>
+        <v>365</v>
       </c>
       <c r="E4" s="40">
         <f>SUM(C4:D4)</f>
-        <v>385</v>
+        <v>425</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="7"/>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="C5" s="58" t="s">
+      <c r="C5" s="62" t="s">
         <v>16</v>
       </c>
-      <c r="D5" s="58"/>
+      <c r="D5" s="62"/>
     </row>
     <row r="6" spans="1:15" s="20" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="18" t="s">
@@ -2675,11 +2696,15 @@
         <v/>
       </c>
       <c r="B26" s="46"/>
-      <c r="C26" s="59"/>
-      <c r="D26" s="60"/>
-      <c r="E26" s="61"/>
-      <c r="F26" s="62"/>
-      <c r="G26" s="55"/>
+      <c r="C26" s="57"/>
+      <c r="D26" s="58"/>
+      <c r="E26" s="59" t="s">
+        <v>58</v>
+      </c>
+      <c r="F26" s="60"/>
+      <c r="G26" s="55" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27" s="16" t="str">
@@ -2687,35 +2712,59 @@
         <v/>
       </c>
       <c r="B27" s="50"/>
-      <c r="C27" s="59"/>
-      <c r="D27" s="60"/>
-      <c r="E27" s="61"/>
-      <c r="F27" s="62"/>
-      <c r="G27" s="56"/>
+      <c r="C27" s="57"/>
+      <c r="D27" s="58"/>
+      <c r="E27" s="59" t="s">
+        <v>58</v>
+      </c>
+      <c r="F27" s="60"/>
+      <c r="G27" s="56" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A28" s="8" t="str">
+      <c r="A28" s="8">
         <f>IF(ISBLANK(B28),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B28))</f>
-        <v/>
-      </c>
-      <c r="B28" s="46"/>
+        <v>19</v>
+      </c>
+      <c r="B28" s="46">
+        <v>45783</v>
+      </c>
       <c r="C28" s="47"/>
-      <c r="D28" s="48"/>
-      <c r="E28" s="49"/>
-      <c r="F28" s="35"/>
-      <c r="G28" s="55"/>
+      <c r="D28" s="48">
+        <v>40</v>
+      </c>
+      <c r="E28" s="49" t="s">
+        <v>4</v>
+      </c>
+      <c r="F28" s="35" t="s">
+        <v>53</v>
+      </c>
+      <c r="G28" s="55" t="s">
+        <v>56</v>
+      </c>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A29" s="16" t="str">
+      <c r="A29" s="16">
         <f>IF(ISBLANK(B29),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B29))</f>
-        <v/>
-      </c>
-      <c r="B29" s="50"/>
+        <v>19</v>
+      </c>
+      <c r="B29" s="50">
+        <v>45783</v>
+      </c>
       <c r="C29" s="51"/>
-      <c r="D29" s="52"/>
-      <c r="E29" s="53"/>
-      <c r="F29" s="35"/>
-      <c r="G29" s="56"/>
+      <c r="D29" s="52" t="s">
+        <v>54</v>
+      </c>
+      <c r="E29" s="53" t="s">
+        <v>4</v>
+      </c>
+      <c r="F29" s="35" t="s">
+        <v>59</v>
+      </c>
+      <c r="G29" s="56" t="s">
+        <v>55</v>
+      </c>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30" s="8" t="str">
@@ -8760,28 +8809,28 @@
     <mergeCell ref="C5:D5"/>
   </mergeCells>
   <conditionalFormatting sqref="E28:E532 E7:E25">
-    <cfRule type="expression" dxfId="7" priority="1">
+    <cfRule type="expression" dxfId="16" priority="1">
       <formula>$E7="Autre"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="6" priority="2" stopIfTrue="1">
+    <cfRule type="expression" dxfId="15" priority="2" stopIfTrue="1">
       <formula>$E7="Design"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="5" priority="3" stopIfTrue="1">
+    <cfRule type="expression" dxfId="14" priority="3" stopIfTrue="1">
       <formula>$E7="Présentation"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="4" stopIfTrue="1">
+    <cfRule type="expression" dxfId="13" priority="4" stopIfTrue="1">
       <formula>$E7="Meeting"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="5" stopIfTrue="1">
+    <cfRule type="expression" dxfId="12" priority="5" stopIfTrue="1">
       <formula>$E7="Documentation"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="2" priority="6" stopIfTrue="1">
+    <cfRule type="expression" dxfId="11" priority="6" stopIfTrue="1">
       <formula>$E7="Test"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="7" stopIfTrue="1">
+    <cfRule type="expression" dxfId="10" priority="7" stopIfTrue="1">
       <formula>$E7="Analyse"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="9" stopIfTrue="1">
+    <cfRule type="expression" dxfId="9" priority="9" stopIfTrue="1">
       <formula>$E7="Développement"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -8854,7 +8903,7 @@
       </c>
       <c r="B5">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Analyse!C5,'Journal de travail'!$D$7:$D$532)</f>
-        <v>130</v>
+        <v>170</v>
       </c>
       <c r="C5" s="41" t="str">
         <f>'Journal de travail'!M9</f>
@@ -8862,7 +8911,7 @@
       </c>
       <c r="D5" s="33">
         <f t="shared" ref="D5:D11" si="0">(A5+B5)/1440</f>
-        <v>0.13194444444444445</v>
+        <v>0.15972222222222221</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
@@ -8979,7 +9028,7 @@
       </c>
       <c r="D12" s="34">
         <f>SUM(D4:D11)</f>
-        <v>0.26736111111111116</v>
+        <v>0.2951388888888889</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
@@ -9002,6 +9051,17 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="be0d3259-a7ce-4623-88ec-81594dfcbc1c" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="99ffe1f3-7857-457f-add0-5bdef636f38d">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D4F20F00DBE2EE49BE9523363A2DF18B" ma:contentTypeVersion="13" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="313dbdbec26224d1c2bb7e3c488b2a4e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="99ffe1f3-7857-457f-add0-5bdef636f38d" xmlns:ns3="be0d3259-a7ce-4623-88ec-81594dfcbc1c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4739345e3d2c6be79c5ae1a54d02a4a7" ns2:_="" ns3:_="">
     <xsd:import namespace="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
@@ -9224,17 +9284,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="be0d3259-a7ce-4623-88ec-81594dfcbc1c" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="99ffe1f3-7857-457f-add0-5bdef636f38d">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>
@@ -9244,6 +9293,17 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="be0d3259-a7ce-4623-88ec-81594dfcbc1c"/>
+    <ds:schemaRef ds:uri="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F2FB702A-DCBD-43A8-A34C-6000FD8861AD}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -9260,15 +9320,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="be0d3259-a7ce-4623-88ec-81594dfcbc1c"/>
-    <ds:schemaRef ds:uri="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
FOOTER ✅correction du footer et integration correcte dans App.vue
FINAL INSTANCE OF FOOTER [ DON'T TOUCH ]
</commit_message>
<xml_diff>
--- a/documentation/JDT-personal/Journal-de-Travail_NademoYosef.xlsx
+++ b/documentation/JDT-personal/Journal-de-Travail_NademoYosef.xlsx
@@ -8,10 +8,10 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pn25kdv\Documents\GitHub\Passion_lecture_FRONTEND\documentation\JDT-personal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99DC3598-6B09-40B6-B3AD-952C1657E838}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{042EF548-8797-443A-B6FC-AB096756FF14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="Mvap2W10CJFFJsnvkGXSiMLvpngxTMJbJsIKFe7Hzjn0XDcmjGuvBC2FjUCZ/hpRpUhUrG1T4kBlDAIo3yqmSQ==" workbookSaltValue="KXjgXOcsUZI/j7UgPKltzw==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="450" yWindow="1290" windowWidth="24840" windowHeight="12270" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
+    <workbookView xWindow="31890" yWindow="855" windowWidth="24840" windowHeight="12270" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal de travail" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="62">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -221,6 +221,12 @@
   </si>
   <si>
     <t>BackEnd(supprimer un problème avec CORS), installation d paquet npm "cors", importation + autorise toutes les origines; TEST avec des images</t>
+  </si>
+  <si>
+    <t>correction du footer et integration correcte dans App.vue</t>
+  </si>
+  <si>
+    <t>FRONTEND(Footer.vue , App.vue , Acceuil.vue)</t>
   </si>
 </sst>
 </file>
@@ -1165,7 +1171,7 @@
                   <c:v>1.3888888888888888E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.15972222222222221</c:v>
+                  <c:v>0.18055555555555555</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -2143,7 +2149,7 @@
       </c>
       <c r="C3" s="22" t="str">
         <f>INT(E4/1440)&amp;" jours "&amp;INT(MOD(E4/1440,1)*24)&amp;" heurs "&amp;INT(MOD(MOD(E4/1440,1)*24,1)*60)&amp;" minutes"</f>
-        <v>0 jours 7 heurs 5 minutes</v>
+        <v>0 jours 7 heurs 35 minutes</v>
       </c>
       <c r="D3" s="22"/>
       <c r="E3" s="3"/>
@@ -2162,11 +2168,11 @@
       </c>
       <c r="D4" s="22">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>365</v>
+        <v>395</v>
       </c>
       <c r="E4" s="40">
         <f>SUM(C4:D4)</f>
-        <v>425</v>
+        <v>455</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="7"/>
@@ -2767,23 +2773,35 @@
       </c>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A30" s="8" t="str">
+      <c r="A30" s="8">
         <f>IF(ISBLANK(B30),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B30))</f>
-        <v/>
-      </c>
-      <c r="B30" s="46"/>
+        <v>19</v>
+      </c>
+      <c r="B30" s="46">
+        <v>45783</v>
+      </c>
       <c r="C30" s="47"/>
-      <c r="D30" s="48"/>
-      <c r="E30" s="49"/>
-      <c r="F30" s="36"/>
-      <c r="G30" s="55"/>
+      <c r="D30" s="48">
+        <v>30</v>
+      </c>
+      <c r="E30" s="49" t="s">
+        <v>4</v>
+      </c>
+      <c r="F30" s="36" t="s">
+        <v>60</v>
+      </c>
+      <c r="G30" s="55" t="s">
+        <v>61</v>
+      </c>
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A31" s="16" t="str">
+      <c r="A31" s="16">
         <f>IF(ISBLANK(B31),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B31))</f>
-        <v/>
-      </c>
-      <c r="B31" s="50"/>
+        <v>19</v>
+      </c>
+      <c r="B31" s="50">
+        <v>45783</v>
+      </c>
       <c r="C31" s="51"/>
       <c r="D31" s="52"/>
       <c r="E31" s="53"/>
@@ -8903,7 +8921,7 @@
       </c>
       <c r="B5">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Analyse!C5,'Journal de travail'!$D$7:$D$532)</f>
-        <v>170</v>
+        <v>200</v>
       </c>
       <c r="C5" s="41" t="str">
         <f>'Journal de travail'!M9</f>
@@ -8911,7 +8929,7 @@
       </c>
       <c r="D5" s="33">
         <f t="shared" ref="D5:D11" si="0">(A5+B5)/1440</f>
-        <v>0.15972222222222221</v>
+        <v>0.18055555555555555</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
@@ -9028,7 +9046,7 @@
       </c>
       <c r="D12" s="34">
         <f>SUM(D4:D11)</f>
-        <v>0.2951388888888889</v>
+        <v>0.31597222222222221</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
modification de mock-book.js , migration(sequelize.js) , Création des 5 premiers livres dans la base de données avec des images réelles et un contenu cohérent; + JDT
"Lors de l'importation des livres via la fonction importBooks(), les liens vers les images (par exemple, les couvertures) n’étaient pas enregistrés en base de données. Cela provenait du fait que la méthode Book.create() ne recevait pas ces champs lors de l’appel.

Résolution :
J’ai modifié la migration pour inclure les champs nécessaires dans la table Books, notamment ceux liés aux images (ex. : coverImageUrl, thumbnailUrl, etc.).

J’ai ensuite mis à jour la fonction importBooks() pour inclure ces champs lors de l’appel à Book.create()."
</commit_message>
<xml_diff>
--- a/documentation/JDT-personal/Journal-de-Travail_NademoYosef.xlsx
+++ b/documentation/JDT-personal/Journal-de-Travail_NademoYosef.xlsx
@@ -8,10 +8,10 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pn25kdv\Documents\GitHub\Passion_lecture_FRONTEND\documentation\JDT-personal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{042EF548-8797-443A-B6FC-AB096756FF14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA8845EA-8031-4A29-A955-AAFDC9C4E249}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="Mvap2W10CJFFJsnvkGXSiMLvpngxTMJbJsIKFe7Hzjn0XDcmjGuvBC2FjUCZ/hpRpUhUrG1T4kBlDAIo3yqmSQ==" workbookSaltValue="KXjgXOcsUZI/j7UgPKltzw==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="31890" yWindow="855" windowWidth="24840" windowHeight="12270" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal de travail" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="66">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -223,10 +223,35 @@
     <t>BackEnd(supprimer un problème avec CORS), installation d paquet npm "cors", importation + autorise toutes les origines; TEST avec des images</t>
   </si>
   <si>
-    <t>correction du footer et integration correcte dans App.vue</t>
+    <t>FRONTEND(Footer.vue , App.vue , Acceuil.vue)</t>
   </si>
   <si>
-    <t>FRONTEND(Footer.vue , App.vue , Acceuil.vue)</t>
+    <t>correction du footer et integration correcte dans App.vue ; Il y avait des problemes dans la partie du code basique, donc j'ai du tout refaire</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BACKEND(DB -Migration)    mock-book.js  </t>
+  </si>
+  <si>
+    <t>modification de mock-book.js  Création des 5 premiers livres dans la base de données avec des images réelles et un contenu cohérent</t>
+  </si>
+  <si>
+    <t>const createdBook = await Book.create({
+  titre: book.titre,
+  annee_edition: book.annee_edition,
+  nombre_de_page: book.nombre_de_page,
+  category_id: book.category_id,
+  writer_id: book.writer_id,
+  lien_image: book.lien_image,
+  lien_pdf: book.lien_pdf,
+  resume: book.resume,
+  editeur: book.editeur,
+});</t>
+  </si>
+  <si>
+    <t>Lors de l'importation des livres via la fonction importBooks(), les liens vers les images (par exemple, les couvertures) n’étaient pas enregistrés en base de données. Cela provenait du fait que la méthode Book.create() ne recevait pas ces champs lors de l’appel.
+Résolution :
+J’ai modifié la migration pour inclure les champs nécessaires dans la table Books, notamment ceux liés aux images (ex. : coverImageUrl, thumbnailUrl, etc.).
+J’ai ensuite mis à jour la fonction importBooks() pour inclure ces champs lors de l’appel à Book.create().</t>
   </si>
 </sst>
 </file>
@@ -1171,13 +1196,13 @@
                   <c:v>1.3888888888888888E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.18055555555555555</c:v>
+                  <c:v>0.21180555555555555</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1.3888888888888888E-2</c:v>
+                  <c:v>2.7777777777777776E-2</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>2.0833333333333332E-2</c:v>
@@ -2149,7 +2174,7 @@
       </c>
       <c r="C3" s="22" t="str">
         <f>INT(E4/1440)&amp;" jours "&amp;INT(MOD(E4/1440,1)*24)&amp;" heurs "&amp;INT(MOD(MOD(E4/1440,1)*24,1)*60)&amp;" minutes"</f>
-        <v>0 jours 7 heurs 35 minutes</v>
+        <v>0 jours 8 heurs 40 minutes</v>
       </c>
       <c r="D3" s="22"/>
       <c r="E3" s="3"/>
@@ -2168,11 +2193,11 @@
       </c>
       <c r="D4" s="22">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>395</v>
+        <v>460</v>
       </c>
       <c r="E4" s="40">
         <f>SUM(C4:D4)</f>
-        <v>455</v>
+        <v>520</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="7"/>
@@ -2772,7 +2797,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:15" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A30" s="8">
         <f>IF(ISBLANK(B30),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B30))</f>
         <v>19</v>
@@ -2788,10 +2813,10 @@
         <v>4</v>
       </c>
       <c r="F30" s="36" t="s">
+        <v>61</v>
+      </c>
+      <c r="G30" s="55" t="s">
         <v>60</v>
-      </c>
-      <c r="G30" s="55" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.25">
@@ -2803,33 +2828,59 @@
         <v>45783</v>
       </c>
       <c r="C31" s="51"/>
-      <c r="D31" s="52"/>
-      <c r="E31" s="53"/>
-      <c r="F31" s="35"/>
-      <c r="G31" s="56"/>
-    </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A32" s="8" t="str">
+      <c r="D31" s="52">
+        <v>30</v>
+      </c>
+      <c r="E31" s="53" t="s">
+        <v>4</v>
+      </c>
+      <c r="F31" s="35" t="s">
+        <v>63</v>
+      </c>
+      <c r="G31" s="56" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="32" spans="1:15" ht="173.25" x14ac:dyDescent="0.25">
+      <c r="A32" s="8">
         <f>IF(ISBLANK(B32),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B32))</f>
-        <v/>
-      </c>
-      <c r="B32" s="46"/>
+        <v>19</v>
+      </c>
+      <c r="B32" s="46">
+        <v>45783</v>
+      </c>
       <c r="C32" s="47"/>
-      <c r="D32" s="48"/>
-      <c r="E32" s="49"/>
-      <c r="F32" s="36"/>
-      <c r="G32" s="55"/>
+      <c r="D32" s="48">
+        <v>15</v>
+      </c>
+      <c r="E32" s="49" t="s">
+        <v>4</v>
+      </c>
+      <c r="F32" s="36" t="s">
+        <v>65</v>
+      </c>
+      <c r="G32" s="55" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" s="16" t="str">
+      <c r="A33" s="16">
         <f>IF(ISBLANK(B33),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B33))</f>
-        <v/>
-      </c>
-      <c r="B33" s="50"/>
+        <v>19</v>
+      </c>
+      <c r="B33" s="50">
+        <v>45783</v>
+      </c>
       <c r="C33" s="51"/>
-      <c r="D33" s="52"/>
-      <c r="E33" s="53"/>
-      <c r="F33" s="35"/>
+      <c r="D33" s="52">
+        <v>20</v>
+      </c>
+      <c r="E33" s="53" t="s">
+        <v>6</v>
+      </c>
+      <c r="F33" s="35" t="s">
+        <v>47</v>
+      </c>
       <c r="G33" s="56"/>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
@@ -8921,7 +8972,7 @@
       </c>
       <c r="B5">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Analyse!C5,'Journal de travail'!$D$7:$D$532)</f>
-        <v>200</v>
+        <v>245</v>
       </c>
       <c r="C5" s="41" t="str">
         <f>'Journal de travail'!M9</f>
@@ -8929,7 +8980,7 @@
       </c>
       <c r="D5" s="33">
         <f t="shared" ref="D5:D11" si="0">(A5+B5)/1440</f>
-        <v>0.18055555555555555</v>
+        <v>0.21180555555555555</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
@@ -8957,7 +9008,7 @@
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Analyse!C7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="C7" s="27" t="str">
         <f>'Journal de travail'!M11</f>
@@ -8965,7 +9016,7 @@
       </c>
       <c r="D7" s="33">
         <f t="shared" si="0"/>
-        <v>1.3888888888888888E-2</v>
+        <v>2.7777777777777776E-2</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
@@ -9046,7 +9097,7 @@
       </c>
       <c r="D12" s="34">
         <f>SUM(D4:D11)</f>
-        <v>0.31597222222222221</v>
+        <v>0.36111111111111105</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Page d'accueil Fonctionnalités globaux [DONE]✅
adaptation des image des livres avec CSS
</commit_message>
<xml_diff>
--- a/documentation/JDT-personal/Journal-de-Travail_NademoYosef.xlsx
+++ b/documentation/JDT-personal/Journal-de-Travail_NademoYosef.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pn25kdv\Documents\GitHub\Passion_lecture_FRONTEND\documentation\JDT-personal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA8845EA-8031-4A29-A955-AAFDC9C4E249}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{435799EB-7811-4BD3-9D5A-5C7B5DD1502D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="Mvap2W10CJFFJsnvkGXSiMLvpngxTMJbJsIKFe7Hzjn0XDcmjGuvBC2FjUCZ/hpRpUhUrG1T4kBlDAIo3yqmSQ==" workbookSaltValue="KXjgXOcsUZI/j7UgPKltzw==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="67">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -252,6 +252,9 @@
 Résolution :
 J’ai modifié la migration pour inclure les champs nécessaires dans la table Books, notamment ceux liés aux images (ex. : coverImageUrl, thumbnailUrl, etc.).
 J’ai ensuite mis à jour la fonction importBooks() pour inclure ces champs lors de l’appel à Book.create().</t>
+  </si>
+  <si>
+    <t>adaptation des image des livres avec CSS</t>
   </si>
 </sst>
 </file>
@@ -1196,7 +1199,7 @@
                   <c:v>1.3888888888888888E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.21180555555555555</c:v>
+                  <c:v>0.21875</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -2174,7 +2177,7 @@
       </c>
       <c r="C3" s="22" t="str">
         <f>INT(E4/1440)&amp;" jours "&amp;INT(MOD(E4/1440,1)*24)&amp;" heurs "&amp;INT(MOD(MOD(E4/1440,1)*24,1)*60)&amp;" minutes"</f>
-        <v>0 jours 8 heurs 40 minutes</v>
+        <v>0 jours 8 heurs 50 minutes</v>
       </c>
       <c r="D3" s="22"/>
       <c r="E3" s="3"/>
@@ -2193,11 +2196,11 @@
       </c>
       <c r="D4" s="22">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>460</v>
+        <v>470</v>
       </c>
       <c r="E4" s="40">
         <f>SUM(C4:D4)</f>
-        <v>520</v>
+        <v>530</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="7"/>
@@ -2873,26 +2876,36 @@
       </c>
       <c r="C33" s="51"/>
       <c r="D33" s="52">
+        <v>10</v>
+      </c>
+      <c r="E33" s="53" t="s">
+        <v>4</v>
+      </c>
+      <c r="F33" s="35" t="s">
+        <v>66</v>
+      </c>
+      <c r="G33" s="56" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34" s="8">
+        <f>IF(ISBLANK(B34),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B34))</f>
+        <v>19</v>
+      </c>
+      <c r="B34" s="46">
+        <v>45783</v>
+      </c>
+      <c r="C34" s="47"/>
+      <c r="D34" s="48">
         <v>20</v>
       </c>
-      <c r="E33" s="53" t="s">
+      <c r="E34" s="49" t="s">
         <v>6</v>
       </c>
-      <c r="F33" s="35" t="s">
+      <c r="F34" s="35" t="s">
         <v>47</v>
       </c>
-      <c r="G33" s="56"/>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A34" s="8" t="str">
-        <f>IF(ISBLANK(B34),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B34))</f>
-        <v/>
-      </c>
-      <c r="B34" s="46"/>
-      <c r="C34" s="47"/>
-      <c r="D34" s="48"/>
-      <c r="E34" s="49"/>
-      <c r="F34" s="35"/>
       <c r="G34" s="55"/>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
@@ -8972,7 +8985,7 @@
       </c>
       <c r="B5">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Analyse!C5,'Journal de travail'!$D$7:$D$532)</f>
-        <v>245</v>
+        <v>255</v>
       </c>
       <c r="C5" s="41" t="str">
         <f>'Journal de travail'!M9</f>
@@ -8980,7 +8993,7 @@
       </c>
       <c r="D5" s="33">
         <f t="shared" ref="D5:D11" si="0">(A5+B5)/1440</f>
-        <v>0.21180555555555555</v>
+        <v>0.21875</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
@@ -9097,7 +9110,7 @@
       </c>
       <c r="D12" s="34">
         <f>SUM(D4:D11)</f>
-        <v>0.36111111111111105</v>
+        <v>0.36805555555555558</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
PageAcceuil lissez la description
PageAcceuil( j'ai fait limitation des livres à 5) + ajuster la taille des images + placement jolie et structurisé sur la page ; PageAcceuil( Title et description ) + ajout de founction showAll pour donner la posibilite de montrer tous les livres ou juste 5 premiers + modification des titres et du text explicatif + (CSS) pour chque de ces étap, transformation des "px" en "em" pour faire un design responsive ; App.vue (CSS)
</commit_message>
<xml_diff>
--- a/documentation/JDT-personal/Journal-de-Travail_NademoYosef.xlsx
+++ b/documentation/JDT-personal/Journal-de-Travail_NademoYosef.xlsx
@@ -8,10 +8,10 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pn25kdv\Documents\GitHub\Passion_lecture_FRONTEND\documentation\JDT-personal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{435799EB-7811-4BD3-9D5A-5C7B5DD1502D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1ABC3B42-3B08-4B59-ACD8-701FC43316F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="Mvap2W10CJFFJsnvkGXSiMLvpngxTMJbJsIKFe7Hzjn0XDcmjGuvBC2FjUCZ/hpRpUhUrG1T4kBlDAIo3yqmSQ==" workbookSaltValue="KXjgXOcsUZI/j7UgPKltzw==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
+    <workbookView xWindow="0" yWindow="705" windowWidth="20700" windowHeight="12270" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal de travail" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="71">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -220,9 +220,6 @@
     <t>ce champs est pas au norme(la partie "Activite")</t>
   </si>
   <si>
-    <t>BackEnd(supprimer un problème avec CORS), installation d paquet npm "cors", importation + autorise toutes les origines; TEST avec des images</t>
-  </si>
-  <si>
     <t>FRONTEND(Footer.vue , App.vue , Acceuil.vue)</t>
   </si>
   <si>
@@ -255,6 +252,25 @@
   </si>
   <si>
     <t>adaptation des image des livres avec CSS</t>
+  </si>
+  <si>
+    <t>BackEnd(supprimer un problème avec CORS), installation de paquet npm "cors", importation + autorise toutes les origines; TEST avec des images</t>
+  </si>
+  <si>
+    <t>&lt;div v-for="book in books.slice(0, 5)" :key="book.livre_id" class="book-card"&gt;</t>
+  </si>
+  <si>
+    <t>PageAcceuil( j'ai fait limitation des livres à 5) + ajuster la taille des images + placement jolie et structurisé sur la page</t>
+  </si>
+  <si>
+    <t>&lt;div
+          v-for="book in showAll ? books : books.slice(0, 5)"
+          :key="book.livre_id"
+          class="book-card"
+        &gt;</t>
+  </si>
+  <si>
+    <t>PageAcceuil( Title et description ) + ajout de founction showAll pour donner la posibilite de montrer tous les livres ou juste 5 premiers + modification des titres et du text explicatif + (CSS) pour chque de ces étap, transformation des "px" en "em" pour faire un design responsive ; App.vue (CSS)</t>
   </si>
 </sst>
 </file>
@@ -1199,7 +1215,7 @@
                   <c:v>1.3888888888888888E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.21875</c:v>
+                  <c:v>0.30208333333333331</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -2177,7 +2193,7 @@
       </c>
       <c r="C3" s="22" t="str">
         <f>INT(E4/1440)&amp;" jours "&amp;INT(MOD(E4/1440,1)*24)&amp;" heurs "&amp;INT(MOD(MOD(E4/1440,1)*24,1)*60)&amp;" minutes"</f>
-        <v>0 jours 8 heurs 50 minutes</v>
+        <v>0 jours 10 heurs 50 minutes</v>
       </c>
       <c r="D3" s="22"/>
       <c r="E3" s="3"/>
@@ -2192,15 +2208,15 @@
       <c r="B4" s="5"/>
       <c r="C4" s="22">
         <f>SUBTOTAL(9,$C$7:$C$531)*60</f>
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="D4" s="22">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>470</v>
+        <v>530</v>
       </c>
       <c r="E4" s="40">
         <f>SUM(C4:D4)</f>
-        <v>530</v>
+        <v>650</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="7"/>
@@ -2794,7 +2810,7 @@
         <v>4</v>
       </c>
       <c r="F29" s="35" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="G29" s="56" t="s">
         <v>55</v>
@@ -2816,10 +2832,10 @@
         <v>4</v>
       </c>
       <c r="F30" s="36" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G30" s="55" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.25">
@@ -2838,10 +2854,10 @@
         <v>4</v>
       </c>
       <c r="F31" s="35" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G31" s="56" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="32" spans="1:15" ht="173.25" x14ac:dyDescent="0.25">
@@ -2860,10 +2876,10 @@
         <v>4</v>
       </c>
       <c r="F32" s="36" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G32" s="55" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
@@ -2882,7 +2898,7 @@
         <v>4</v>
       </c>
       <c r="F33" s="35" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G33" s="56" t="s">
         <v>56</v>
@@ -2908,29 +2924,51 @@
       </c>
       <c r="G34" s="55"/>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A35" s="16" t="str">
+    <row r="35" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A35" s="16">
         <f>IF(ISBLANK(B35),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B35))</f>
-        <v/>
-      </c>
-      <c r="B35" s="50"/>
+        <v>19</v>
+      </c>
+      <c r="B35" s="50">
+        <v>45784</v>
+      </c>
       <c r="C35" s="51"/>
-      <c r="D35" s="52"/>
-      <c r="E35" s="53"/>
-      <c r="F35" s="36"/>
-      <c r="G35" s="56"/>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A36" s="8" t="str">
+      <c r="D35" s="52">
+        <v>30</v>
+      </c>
+      <c r="E35" s="53" t="s">
+        <v>4</v>
+      </c>
+      <c r="F35" s="36" t="s">
+        <v>68</v>
+      </c>
+      <c r="G35" s="56" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" ht="78.75" x14ac:dyDescent="0.25">
+      <c r="A36" s="8">
         <f>IF(ISBLANK(B36),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B36))</f>
-        <v/>
-      </c>
-      <c r="B36" s="46"/>
-      <c r="C36" s="47"/>
-      <c r="D36" s="48"/>
-      <c r="E36" s="49"/>
-      <c r="F36" s="35"/>
-      <c r="G36" s="55"/>
+        <v>19</v>
+      </c>
+      <c r="B36" s="46">
+        <v>45784</v>
+      </c>
+      <c r="C36" s="47">
+        <v>1</v>
+      </c>
+      <c r="D36" s="48">
+        <v>30</v>
+      </c>
+      <c r="E36" s="49" t="s">
+        <v>4</v>
+      </c>
+      <c r="F36" s="35" t="s">
+        <v>70</v>
+      </c>
+      <c r="G36" s="55" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="16" t="str">
@@ -8981,11 +9019,11 @@
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Analyse!C5,'Journal de travail'!$C$7:$C$532)*60</f>
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="B5">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Analyse!C5,'Journal de travail'!$D$7:$D$532)</f>
-        <v>255</v>
+        <v>315</v>
       </c>
       <c r="C5" s="41" t="str">
         <f>'Journal de travail'!M9</f>
@@ -8993,7 +9031,7 @@
       </c>
       <c r="D5" s="33">
         <f t="shared" ref="D5:D11" si="0">(A5+B5)/1440</f>
-        <v>0.21875</v>
+        <v>0.30208333333333331</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
@@ -9110,7 +9148,7 @@
       </c>
       <c r="D12" s="34">
         <f>SUM(D4:D11)</f>
-        <v>0.36805555555555558</v>
+        <v>0.45138888888888884</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
@@ -9133,17 +9171,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="be0d3259-a7ce-4623-88ec-81594dfcbc1c" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="99ffe1f3-7857-457f-add0-5bdef636f38d">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D4F20F00DBE2EE49BE9523363A2DF18B" ma:contentTypeVersion="13" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="313dbdbec26224d1c2bb7e3c488b2a4e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="99ffe1f3-7857-457f-add0-5bdef636f38d" xmlns:ns3="be0d3259-a7ce-4623-88ec-81594dfcbc1c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4739345e3d2c6be79c5ae1a54d02a4a7" ns2:_="" ns3:_="">
     <xsd:import namespace="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
@@ -9366,6 +9393,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="be0d3259-a7ce-4623-88ec-81594dfcbc1c" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="99ffe1f3-7857-457f-add0-5bdef636f38d">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>
@@ -9375,17 +9413,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="be0d3259-a7ce-4623-88ec-81594dfcbc1c"/>
-    <ds:schemaRef ds:uri="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F2FB702A-DCBD-43A8-A34C-6000FD8861AD}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -9402,4 +9429,15 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="be0d3259-a7ce-4623-88ec-81594dfcbc1c"/>
+    <ds:schemaRef ds:uri="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Création de css pour la page des livres d'une "category"✅ ;  Création de css pour la page des categories ✅
Création de css pour la page des livres d'une "category"✅ ;  Création de css pour la page des categories ✅ + JDT
</commit_message>
<xml_diff>
--- a/documentation/JDT-personal/Journal-de-Travail_NademoYosef.xlsx
+++ b/documentation/JDT-personal/Journal-de-Travail_NademoYosef.xlsx
@@ -8,10 +8,10 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pn25kdv\Documents\GitHub\Passion_lecture_FRONTEND\documentation\JDT-personal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1ABC3B42-3B08-4B59-ACD8-701FC43316F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F3BA330-6C1B-4DDD-A606-BFFBB34C20CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="Mvap2W10CJFFJsnvkGXSiMLvpngxTMJbJsIKFe7Hzjn0XDcmjGuvBC2FjUCZ/hpRpUhUrG1T4kBlDAIo3yqmSQ==" workbookSaltValue="KXjgXOcsUZI/j7UgPKltzw==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="705" windowWidth="20700" windowHeight="12270" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
+    <workbookView xWindow="32355" yWindow="0" windowWidth="23520" windowHeight="15600" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal de travail" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="73">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -271,6 +271,12 @@
   </si>
   <si>
     <t>PageAcceuil( Title et description ) + ajout de founction showAll pour donner la posibilite de montrer tous les livres ou juste 5 premiers + modification des titres et du text explicatif + (CSS) pour chque de ces étap, transformation des "px" en "em" pour faire un design responsive ; App.vue (CSS)</t>
+  </si>
+  <si>
+    <t>Création de css pour la page des categories</t>
+  </si>
+  <si>
+    <t>Création de css pour la page des livres d'une "category"</t>
   </si>
 </sst>
 </file>
@@ -1215,13 +1221,13 @@
                   <c:v>1.3888888888888888E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.30208333333333331</c:v>
+                  <c:v>0.34375</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2.7777777777777776E-2</c:v>
+                  <c:v>4.1666666666666664E-2</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>2.0833333333333332E-2</c:v>
@@ -2193,7 +2199,7 @@
       </c>
       <c r="C3" s="22" t="str">
         <f>INT(E4/1440)&amp;" jours "&amp;INT(MOD(E4/1440,1)*24)&amp;" heurs "&amp;INT(MOD(MOD(E4/1440,1)*24,1)*60)&amp;" minutes"</f>
-        <v>0 jours 10 heurs 50 minutes</v>
+        <v>0 jours 12 heurs 9 minutes</v>
       </c>
       <c r="D3" s="22"/>
       <c r="E3" s="3"/>
@@ -2212,11 +2218,11 @@
       </c>
       <c r="D4" s="22">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>530</v>
+        <v>610</v>
       </c>
       <c r="E4" s="40">
         <f>SUM(C4:D4)</f>
-        <v>650</v>
+        <v>730</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="7"/>
@@ -2971,39 +2977,63 @@
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A37" s="16" t="str">
+      <c r="A37" s="16">
         <f>IF(ISBLANK(B37),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B37))</f>
-        <v/>
-      </c>
-      <c r="B37" s="50"/>
+        <v>19</v>
+      </c>
+      <c r="B37" s="50">
+        <v>45784</v>
+      </c>
       <c r="C37" s="51"/>
-      <c r="D37" s="52"/>
-      <c r="E37" s="53"/>
-      <c r="F37" s="35"/>
+      <c r="D37" s="52">
+        <v>30</v>
+      </c>
+      <c r="E37" s="53" t="s">
+        <v>4</v>
+      </c>
+      <c r="F37" s="35" t="s">
+        <v>71</v>
+      </c>
       <c r="G37" s="56"/>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A38" s="8" t="str">
+      <c r="A38" s="8">
         <f>IF(ISBLANK(B38),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B38))</f>
-        <v/>
-      </c>
-      <c r="B38" s="46"/>
+        <v>19</v>
+      </c>
+      <c r="B38" s="46">
+        <v>45784</v>
+      </c>
       <c r="C38" s="47"/>
-      <c r="D38" s="48"/>
-      <c r="E38" s="49"/>
-      <c r="F38" s="35"/>
+      <c r="D38" s="48">
+        <v>30</v>
+      </c>
+      <c r="E38" s="49" t="s">
+        <v>4</v>
+      </c>
+      <c r="F38" s="35" t="s">
+        <v>72</v>
+      </c>
       <c r="G38" s="55"/>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A39" s="16" t="str">
+      <c r="A39" s="16">
         <f>IF(ISBLANK(B39),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B39))</f>
-        <v/>
-      </c>
-      <c r="B39" s="50"/>
+        <v>19</v>
+      </c>
+      <c r="B39" s="50">
+        <v>45784</v>
+      </c>
       <c r="C39" s="51"/>
-      <c r="D39" s="52"/>
-      <c r="E39" s="53"/>
-      <c r="F39" s="35"/>
+      <c r="D39" s="52">
+        <v>20</v>
+      </c>
+      <c r="E39" s="53" t="s">
+        <v>6</v>
+      </c>
+      <c r="F39" s="35" t="s">
+        <v>47</v>
+      </c>
       <c r="G39" s="56"/>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
@@ -9023,7 +9053,7 @@
       </c>
       <c r="B5">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Analyse!C5,'Journal de travail'!$D$7:$D$532)</f>
-        <v>315</v>
+        <v>375</v>
       </c>
       <c r="C5" s="41" t="str">
         <f>'Journal de travail'!M9</f>
@@ -9031,7 +9061,7 @@
       </c>
       <c r="D5" s="33">
         <f t="shared" ref="D5:D11" si="0">(A5+B5)/1440</f>
-        <v>0.30208333333333331</v>
+        <v>0.34375</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
@@ -9059,7 +9089,7 @@
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Analyse!C7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="C7" s="27" t="str">
         <f>'Journal de travail'!M11</f>
@@ -9067,7 +9097,7 @@
       </c>
       <c r="D7" s="33">
         <f t="shared" si="0"/>
-        <v>2.7777777777777776E-2</v>
+        <v>4.1666666666666664E-2</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
@@ -9148,7 +9178,7 @@
       </c>
       <c r="D12" s="34">
         <f>SUM(D4:D11)</f>
-        <v>0.45138888888888884</v>
+        <v>0.50694444444444442</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
CSS pour une page d’ajout d’un ouvrage (accès utilisateur)
 CSS pour une page d’ajout d’un ouvrage (accès utilisateur)  + JDT
</commit_message>
<xml_diff>
--- a/documentation/JDT-personal/Journal-de-Travail_NademoYosef.xlsx
+++ b/documentation/JDT-personal/Journal-de-Travail_NademoYosef.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pn25kdv\Documents\GitHub\Passion_lecture_FRONTEND\documentation\JDT-personal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{378A9821-98DE-44A0-9A60-55F73B979D31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F15DBC02-A812-42E1-BAA6-9CAD6E33849C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="Mvap2W10CJFFJsnvkGXSiMLvpngxTMJbJsIKFe7Hzjn0XDcmjGuvBC2FjUCZ/hpRpUhUrG1T4kBlDAIo3yqmSQ==" workbookSaltValue="KXjgXOcsUZI/j7UgPKltzw==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
     <workbookView xWindow="4320" yWindow="765" windowWidth="23520" windowHeight="14235" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="76">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -283,6 +283,10 @@
   </si>
   <si>
     <t>Page d'ajout d'un ouvrage (transfering data vers API et db)script; utilisation le user qui est dans JWT token, creation de methode</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+CSS pour une page d’ajout d’un ouvrage (accès utilisateur)</t>
   </si>
 </sst>
 </file>
@@ -1227,7 +1231,7 @@
                   <c:v>1.3888888888888888E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.4201388888888889</c:v>
+                  <c:v>0.44097222222222221</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -2205,7 +2209,7 @@
       </c>
       <c r="C3" s="22" t="str">
         <f>INT(E4/1440)&amp;" jours "&amp;INT(MOD(E4/1440,1)*24)&amp;" heurs "&amp;INT(MOD(MOD(E4/1440,1)*24,1)*60)&amp;" minutes"</f>
-        <v>0 jours 14 heurs 0 minutes</v>
+        <v>0 jours 14 heurs 30 minutes</v>
       </c>
       <c r="D3" s="22"/>
       <c r="E3" s="3"/>
@@ -2224,11 +2228,11 @@
       </c>
       <c r="D4" s="22">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>660</v>
+        <v>690</v>
       </c>
       <c r="E4" s="40">
         <f>SUM(C4:D4)</f>
-        <v>840</v>
+        <v>870</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="7"/>
@@ -3084,16 +3088,24 @@
       </c>
       <c r="G41" s="56"/>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A42" s="8" t="str">
+    <row r="42" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A42" s="8">
         <f>IF(ISBLANK(B42),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B42))</f>
-        <v/>
-      </c>
-      <c r="B42" s="46"/>
+        <v>20</v>
+      </c>
+      <c r="B42" s="46">
+        <v>45790</v>
+      </c>
       <c r="C42" s="47"/>
-      <c r="D42" s="48"/>
-      <c r="E42" s="49"/>
-      <c r="F42" s="35"/>
+      <c r="D42" s="48">
+        <v>30</v>
+      </c>
+      <c r="E42" s="49" t="s">
+        <v>4</v>
+      </c>
+      <c r="F42" s="36" t="s">
+        <v>75</v>
+      </c>
       <c r="G42" s="55"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
@@ -9077,7 +9089,7 @@
       </c>
       <c r="B5">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Analyse!C5,'Journal de travail'!$D$7:$D$532)</f>
-        <v>425</v>
+        <v>455</v>
       </c>
       <c r="C5" s="41" t="str">
         <f>'Journal de travail'!M9</f>
@@ -9085,7 +9097,7 @@
       </c>
       <c r="D5" s="33">
         <f t="shared" ref="D5:D11" si="0">(A5+B5)/1440</f>
-        <v>0.4201388888888889</v>
+        <v>0.44097222222222221</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
@@ -9202,7 +9214,7 @@
       </c>
       <c r="D12" s="34">
         <f>SUM(D4:D11)</f>
-        <v>0.58333333333333337</v>
+        <v>0.60416666666666674</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
@@ -9225,6 +9237,17 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="be0d3259-a7ce-4623-88ec-81594dfcbc1c" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="99ffe1f3-7857-457f-add0-5bdef636f38d">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D4F20F00DBE2EE49BE9523363A2DF18B" ma:contentTypeVersion="13" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="313dbdbec26224d1c2bb7e3c488b2a4e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="99ffe1f3-7857-457f-add0-5bdef636f38d" xmlns:ns3="be0d3259-a7ce-4623-88ec-81594dfcbc1c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4739345e3d2c6be79c5ae1a54d02a4a7" ns2:_="" ns3:_="">
     <xsd:import namespace="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
@@ -9447,17 +9470,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="be0d3259-a7ce-4623-88ec-81594dfcbc1c" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="99ffe1f3-7857-457f-add0-5bdef636f38d">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>
@@ -9467,6 +9479,17 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="be0d3259-a7ce-4623-88ec-81594dfcbc1c"/>
+    <ds:schemaRef ds:uri="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F2FB702A-DCBD-43A8-A34C-6000FD8861AD}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -9483,15 +9506,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="be0d3259-a7ce-4623-88ec-81594dfcbc1c"/>
-    <ds:schemaRef ds:uri="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
creation du methode qui gere ajouter des images +jdt
</commit_message>
<xml_diff>
--- a/documentation/JDT-personal/Journal-de-Travail_NademoYosef.xlsx
+++ b/documentation/JDT-personal/Journal-de-Travail_NademoYosef.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pn25kdv\Documents\GitHub\Passion_lecture_FRONTEND\documentation\JDT-personal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F15DBC02-A812-42E1-BAA6-9CAD6E33849C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CBA4C3B-A56B-4F7F-9397-668BB45DD1BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="Mvap2W10CJFFJsnvkGXSiMLvpngxTMJbJsIKFe7Hzjn0XDcmjGuvBC2FjUCZ/hpRpUhUrG1T4kBlDAIo3yqmSQ==" workbookSaltValue="KXjgXOcsUZI/j7UgPKltzw==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
     <workbookView xWindow="4320" yWindow="765" windowWidth="23520" windowHeight="14235" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="77">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -287,6 +287,9 @@
   <si>
     <t xml:space="preserve">
 CSS pour une page d’ajout d’un ouvrage (accès utilisateur)</t>
+  </si>
+  <si>
+    <t>creation du methode qui gere ajouter des images</t>
   </si>
 </sst>
 </file>
@@ -1231,7 +1234,7 @@
                   <c:v>1.3888888888888888E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.44097222222222221</c:v>
+                  <c:v>0.46180555555555558</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -2209,7 +2212,7 @@
       </c>
       <c r="C3" s="22" t="str">
         <f>INT(E4/1440)&amp;" jours "&amp;INT(MOD(E4/1440,1)*24)&amp;" heurs "&amp;INT(MOD(MOD(E4/1440,1)*24,1)*60)&amp;" minutes"</f>
-        <v>0 jours 14 heurs 30 minutes</v>
+        <v>0 jours 15 heurs 0 minutes</v>
       </c>
       <c r="D3" s="22"/>
       <c r="E3" s="3"/>
@@ -2228,11 +2231,11 @@
       </c>
       <c r="D4" s="22">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>690</v>
+        <v>720</v>
       </c>
       <c r="E4" s="40">
         <f>SUM(C4:D4)</f>
-        <v>870</v>
+        <v>900</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="7"/>
@@ -3109,15 +3112,23 @@
       <c r="G42" s="55"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A43" s="16" t="str">
+      <c r="A43" s="16">
         <f>IF(ISBLANK(B43),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B43))</f>
-        <v/>
-      </c>
-      <c r="B43" s="50"/>
+        <v>20</v>
+      </c>
+      <c r="B43" s="50">
+        <v>45790</v>
+      </c>
       <c r="C43" s="51"/>
-      <c r="D43" s="52"/>
-      <c r="E43" s="53"/>
-      <c r="F43" s="35"/>
+      <c r="D43" s="52">
+        <v>30</v>
+      </c>
+      <c r="E43" s="53" t="s">
+        <v>4</v>
+      </c>
+      <c r="F43" s="35" t="s">
+        <v>76</v>
+      </c>
       <c r="G43" s="56"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
@@ -9089,7 +9100,7 @@
       </c>
       <c r="B5">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Analyse!C5,'Journal de travail'!$D$7:$D$532)</f>
-        <v>455</v>
+        <v>485</v>
       </c>
       <c r="C5" s="41" t="str">
         <f>'Journal de travail'!M9</f>
@@ -9097,7 +9108,7 @@
       </c>
       <c r="D5" s="33">
         <f t="shared" ref="D5:D11" si="0">(A5+B5)/1440</f>
-        <v>0.44097222222222221</v>
+        <v>0.46180555555555558</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
@@ -9214,7 +9225,7 @@
       </c>
       <c r="D12" s="34">
         <f>SUM(D4:D11)</f>
-        <v>0.60416666666666674</v>
+        <v>0.62500000000000011</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
@@ -9237,17 +9248,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="be0d3259-a7ce-4623-88ec-81594dfcbc1c" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="99ffe1f3-7857-457f-add0-5bdef636f38d">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D4F20F00DBE2EE49BE9523363A2DF18B" ma:contentTypeVersion="13" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="313dbdbec26224d1c2bb7e3c488b2a4e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="99ffe1f3-7857-457f-add0-5bdef636f38d" xmlns:ns3="be0d3259-a7ce-4623-88ec-81594dfcbc1c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4739345e3d2c6be79c5ae1a54d02a4a7" ns2:_="" ns3:_="">
     <xsd:import namespace="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
@@ -9470,6 +9470,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="be0d3259-a7ce-4623-88ec-81594dfcbc1c" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="99ffe1f3-7857-457f-add0-5bdef636f38d">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>
@@ -9479,17 +9490,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="be0d3259-a7ce-4623-88ec-81594dfcbc1c"/>
-    <ds:schemaRef ds:uri="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F2FB702A-DCBD-43A8-A34C-6000FD8861AD}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -9506,4 +9506,15 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="be0d3259-a7ce-4623-88ec-81594dfcbc1c"/>
+    <ds:schemaRef ds:uri="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Une page d’ajout d’un ouvrage✅
Configuration de multer(pour parce le ficher avec données) upload.js
booksController.js
      // Find or create a writer
      // Find or create a category
      // Create a book
CreateBook.vue
Methode pour resevoir des images depuis une ligne extérieur(URL d'un site externe) , ou depuis le serveur
DOSSIER uploads,qui contien des images charge par utilisateur ,redirection correct vers ce dossier

gitignore
</commit_message>
<xml_diff>
--- a/documentation/JDT-personal/Journal-de-Travail_NademoYosef.xlsx
+++ b/documentation/JDT-personal/Journal-de-Travail_NademoYosef.xlsx
@@ -8,10 +8,10 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pn25kdv\Documents\GitHub\Passion_lecture_FRONTEND\documentation\JDT-personal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CBA4C3B-A56B-4F7F-9397-668BB45DD1BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF2468BA-F699-4E27-A45D-31B0186F1C5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="Mvap2W10CJFFJsnvkGXSiMLvpngxTMJbJsIKFe7Hzjn0XDcmjGuvBC2FjUCZ/hpRpUhUrG1T4kBlDAIo3yqmSQ==" workbookSaltValue="KXjgXOcsUZI/j7UgPKltzw==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="4320" yWindow="765" windowWidth="23520" windowHeight="14235" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
+    <workbookView xWindow="3960" yWindow="540" windowWidth="23520" windowHeight="14235" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal de travail" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="82">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -290,6 +290,31 @@
   </si>
   <si>
     <t>creation du methode qui gere ajouter des images</t>
+  </si>
+  <si>
+    <t>Update README.md Installation et deploiement+ explication du script</t>
+  </si>
+  <si>
+    <t>Script de démarrage automatique✅; docker compose modification suppresion de app (9999)</t>
+  </si>
+  <si>
+    <t>Gain de temps : plus besoin d'explorer chaque dossier, d'exécuter des commandes individuelles ou de réfléchir à l'ordre de lancement.
+- Commodité pour l'équipe : tout développeur peut commencer à travailler rapidement sans comprendre la structure du projet.
+- Fiabilité accrue : le risque d'erreur humaine lors du lancement manuel est réduit.</t>
+  </si>
+  <si>
+    <t>Une page d’ajout d’un ouvrage</t>
+  </si>
+  <si>
+    <t>Configuration de multer(pour parce le ficher avec données) upload.js
+booksController.js
+      // Find or create a writer
+      // Find or create a category
+      // Create a book
+CreateBook.vue
+Methode pour resevoir des images depuis une ligne extérieur(URL d'un site externe) , ou depuis le serveur
+DOSSIER uploads,qui contien des images charge par utilisateur ,redirection correct vers ce dossier
+gitignore</t>
   </si>
 </sst>
 </file>
@@ -1234,13 +1259,13 @@
                   <c:v>1.3888888888888888E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.46180555555555558</c:v>
+                  <c:v>0.56597222222222221</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>4.1666666666666664E-2</c:v>
+                  <c:v>6.25E-2</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>2.0833333333333332E-2</c:v>
@@ -2212,7 +2237,7 @@
       </c>
       <c r="C3" s="22" t="str">
         <f>INT(E4/1440)&amp;" jours "&amp;INT(MOD(E4/1440,1)*24)&amp;" heurs "&amp;INT(MOD(MOD(E4/1440,1)*24,1)*60)&amp;" minutes"</f>
-        <v>0 jours 15 heurs 0 minutes</v>
+        <v>0 jours 18 heurs 0 minutes</v>
       </c>
       <c r="D3" s="22"/>
       <c r="E3" s="3"/>
@@ -2227,15 +2252,15 @@
       <c r="B4" s="5"/>
       <c r="C4" s="22">
         <f>SUBTOTAL(9,$C$7:$C$531)*60</f>
-        <v>180</v>
+        <v>240</v>
       </c>
       <c r="D4" s="22">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>720</v>
+        <v>840</v>
       </c>
       <c r="E4" s="40">
         <f>SUM(C4:D4)</f>
-        <v>900</v>
+        <v>1080</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="7"/>
@@ -3132,40 +3157,70 @@
       <c r="G43" s="56"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A44" s="8" t="str">
+      <c r="A44" s="8">
         <f>IF(ISBLANK(B44),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B44))</f>
-        <v/>
-      </c>
-      <c r="B44" s="46"/>
+        <v>21</v>
+      </c>
+      <c r="B44" s="46">
+        <v>45797</v>
+      </c>
       <c r="C44" s="47"/>
-      <c r="D44" s="48"/>
-      <c r="E44" s="49"/>
-      <c r="F44" s="35"/>
+      <c r="D44" s="48">
+        <v>30</v>
+      </c>
+      <c r="E44" s="49" t="s">
+        <v>6</v>
+      </c>
+      <c r="F44" s="35" t="s">
+        <v>77</v>
+      </c>
       <c r="G44" s="55"/>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A45" s="16" t="str">
+    <row r="45" spans="1:7" ht="110.25" x14ac:dyDescent="0.25">
+      <c r="A45" s="16">
         <f>IF(ISBLANK(B45),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B45))</f>
-        <v/>
-      </c>
-      <c r="B45" s="50"/>
+        <v>21</v>
+      </c>
+      <c r="B45" s="50">
+        <v>45797</v>
+      </c>
       <c r="C45" s="51"/>
-      <c r="D45" s="52"/>
-      <c r="E45" s="53"/>
-      <c r="F45" s="35"/>
-      <c r="G45" s="56"/>
-    </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A46" s="8" t="str">
+      <c r="D45" s="52">
+        <v>40</v>
+      </c>
+      <c r="E45" s="53" t="s">
+        <v>4</v>
+      </c>
+      <c r="F45" s="35" t="s">
+        <v>78</v>
+      </c>
+      <c r="G45" s="56" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" ht="189" x14ac:dyDescent="0.25">
+      <c r="A46" s="8">
         <f>IF(ISBLANK(B46),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B46))</f>
-        <v/>
-      </c>
-      <c r="B46" s="46"/>
-      <c r="C46" s="47"/>
-      <c r="D46" s="48"/>
-      <c r="E46" s="49"/>
-      <c r="F46" s="35"/>
-      <c r="G46" s="55"/>
+        <v>21</v>
+      </c>
+      <c r="B46" s="46">
+        <v>45797</v>
+      </c>
+      <c r="C46" s="47">
+        <v>1</v>
+      </c>
+      <c r="D46" s="48">
+        <v>50</v>
+      </c>
+      <c r="E46" s="49" t="s">
+        <v>4</v>
+      </c>
+      <c r="F46" s="35" t="s">
+        <v>80</v>
+      </c>
+      <c r="G46" s="55" t="s">
+        <v>81</v>
+      </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" s="16" t="str">
@@ -9096,11 +9151,11 @@
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Analyse!C5,'Journal de travail'!$C$7:$C$532)*60</f>
-        <v>180</v>
+        <v>240</v>
       </c>
       <c r="B5">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Analyse!C5,'Journal de travail'!$D$7:$D$532)</f>
-        <v>485</v>
+        <v>575</v>
       </c>
       <c r="C5" s="41" t="str">
         <f>'Journal de travail'!M9</f>
@@ -9108,7 +9163,7 @@
       </c>
       <c r="D5" s="33">
         <f t="shared" ref="D5:D11" si="0">(A5+B5)/1440</f>
-        <v>0.46180555555555558</v>
+        <v>0.56597222222222221</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
@@ -9136,7 +9191,7 @@
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Analyse!C7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="C7" s="27" t="str">
         <f>'Journal de travail'!M11</f>
@@ -9144,7 +9199,7 @@
       </c>
       <c r="D7" s="33">
         <f t="shared" si="0"/>
-        <v>4.1666666666666664E-2</v>
+        <v>6.25E-2</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
@@ -9225,7 +9280,7 @@
       </c>
       <c r="D12" s="34">
         <f>SUM(D4:D11)</f>
-        <v>0.62500000000000011</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
@@ -9248,6 +9303,17 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="be0d3259-a7ce-4623-88ec-81594dfcbc1c" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="99ffe1f3-7857-457f-add0-5bdef636f38d">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D4F20F00DBE2EE49BE9523363A2DF18B" ma:contentTypeVersion="13" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="313dbdbec26224d1c2bb7e3c488b2a4e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="99ffe1f3-7857-457f-add0-5bdef636f38d" xmlns:ns3="be0d3259-a7ce-4623-88ec-81594dfcbc1c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4739345e3d2c6be79c5ae1a54d02a4a7" ns2:_="" ns3:_="">
     <xsd:import namespace="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
@@ -9470,17 +9536,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="be0d3259-a7ce-4623-88ec-81594dfcbc1c" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="99ffe1f3-7857-457f-add0-5bdef636f38d">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>
@@ -9490,6 +9545,17 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="be0d3259-a7ce-4623-88ec-81594dfcbc1c"/>
+    <ds:schemaRef ds:uri="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F2FB702A-DCBD-43A8-A34C-6000FD8861AD}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -9506,15 +9572,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="be0d3259-a7ce-4623-88ec-81594dfcbc1c"/>
-    <ds:schemaRef ds:uri="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Rapport (structure de rapport, WEBOGRAPHIE)
</commit_message>
<xml_diff>
--- a/documentation/JDT-personal/Journal-de-Travail_NademoYosef.xlsx
+++ b/documentation/JDT-personal/Journal-de-Travail_NademoYosef.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pn25kdv\Documents\GitHub\Passion_lecture_FRONTEND\documentation\JDT-personal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF2468BA-F699-4E27-A45D-31B0186F1C5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAF490E3-D14D-47EC-98AA-6C35EE0CE89F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="Mvap2W10CJFFJsnvkGXSiMLvpngxTMJbJsIKFe7Hzjn0XDcmjGuvBC2FjUCZ/hpRpUhUrG1T4kBlDAIo3yqmSQ==" workbookSaltValue="KXjgXOcsUZI/j7UgPKltzw==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
     <workbookView xWindow="3960" yWindow="540" windowWidth="23520" windowHeight="14235" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="83">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -315,6 +315,9 @@
 Methode pour resevoir des images depuis une ligne extérieur(URL d'un site externe) , ou depuis le serveur
 DOSSIER uploads,qui contien des images charge par utilisateur ,redirection correct vers ce dossier
 gitignore</t>
+  </si>
+  <si>
+    <t>Rapport (structure de rapport, WEBOGRAPHIE)</t>
   </si>
 </sst>
 </file>
@@ -1265,7 +1268,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>6.25E-2</c:v>
+                  <c:v>8.3333333333333329E-2</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>2.0833333333333332E-2</c:v>
@@ -2237,7 +2240,7 @@
       </c>
       <c r="C3" s="22" t="str">
         <f>INT(E4/1440)&amp;" jours "&amp;INT(MOD(E4/1440,1)*24)&amp;" heurs "&amp;INT(MOD(MOD(E4/1440,1)*24,1)*60)&amp;" minutes"</f>
-        <v>0 jours 18 heurs 0 minutes</v>
+        <v>0 jours 18 heurs 30 minutes</v>
       </c>
       <c r="D3" s="22"/>
       <c r="E3" s="3"/>
@@ -2256,11 +2259,11 @@
       </c>
       <c r="D4" s="22">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>840</v>
+        <v>870</v>
       </c>
       <c r="E4" s="40">
         <f>SUM(C4:D4)</f>
-        <v>1080</v>
+        <v>1110</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="7"/>
@@ -3223,15 +3226,23 @@
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A47" s="16" t="str">
+      <c r="A47" s="16">
         <f>IF(ISBLANK(B47),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B47))</f>
-        <v/>
-      </c>
-      <c r="B47" s="50"/>
+        <v>21</v>
+      </c>
+      <c r="B47" s="50">
+        <v>45797</v>
+      </c>
       <c r="C47" s="51"/>
-      <c r="D47" s="52"/>
-      <c r="E47" s="53"/>
-      <c r="F47" s="35"/>
+      <c r="D47" s="52">
+        <v>30</v>
+      </c>
+      <c r="E47" s="53" t="s">
+        <v>6</v>
+      </c>
+      <c r="F47" s="35" t="s">
+        <v>82</v>
+      </c>
       <c r="G47" s="56"/>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
@@ -9191,7 +9202,7 @@
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Analyse!C7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>90</v>
+        <v>120</v>
       </c>
       <c r="C7" s="27" t="str">
         <f>'Journal de travail'!M11</f>
@@ -9199,7 +9210,7 @@
       </c>
       <c r="D7" s="33">
         <f t="shared" si="0"/>
-        <v>6.25E-2</v>
+        <v>8.3333333333333329E-2</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
@@ -9280,7 +9291,7 @@
       </c>
       <c r="D12" s="34">
         <f>SUM(D4:D11)</f>
-        <v>0.75</v>
+        <v>0.77083333333333337</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
@@ -9303,17 +9314,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="be0d3259-a7ce-4623-88ec-81594dfcbc1c" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="99ffe1f3-7857-457f-add0-5bdef636f38d">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D4F20F00DBE2EE49BE9523363A2DF18B" ma:contentTypeVersion="13" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="313dbdbec26224d1c2bb7e3c488b2a4e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="99ffe1f3-7857-457f-add0-5bdef636f38d" xmlns:ns3="be0d3259-a7ce-4623-88ec-81594dfcbc1c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4739345e3d2c6be79c5ae1a54d02a4a7" ns2:_="" ns3:_="">
     <xsd:import namespace="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
@@ -9536,6 +9536,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="be0d3259-a7ce-4623-88ec-81594dfcbc1c" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="99ffe1f3-7857-457f-add0-5bdef636f38d">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>
@@ -9545,17 +9556,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="be0d3259-a7ce-4623-88ec-81594dfcbc1c"/>
-    <ds:schemaRef ds:uri="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F2FB702A-DCBD-43A8-A34C-6000FD8861AD}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -9572,4 +9572,15 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="be0d3259-a7ce-4623-88ec-81594dfcbc1c"/>
+    <ds:schemaRef ds:uri="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
rapport (structure ,intorduction,2	ANALYSE 2.1	Planification de toutes les tâches à réaliser Planification des tâches (outil GitHub Projects))
</commit_message>
<xml_diff>
--- a/documentation/JDT-personal/Journal-de-Travail_NademoYosef.xlsx
+++ b/documentation/JDT-personal/Journal-de-Travail_NademoYosef.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pn25kdv\Documents\GitHub\Passion_lecture_FRONTEND\documentation\JDT-personal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAF490E3-D14D-47EC-98AA-6C35EE0CE89F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{116E6EBC-87C9-4839-A4C7-8D10508DE0FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="Mvap2W10CJFFJsnvkGXSiMLvpngxTMJbJsIKFe7Hzjn0XDcmjGuvBC2FjUCZ/hpRpUhUrG1T4kBlDAIo3yqmSQ==" workbookSaltValue="KXjgXOcsUZI/j7UgPKltzw==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
     <workbookView xWindow="3960" yWindow="540" windowWidth="23520" windowHeight="14235" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="84">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -318,6 +318,9 @@
   </si>
   <si>
     <t>Rapport (structure de rapport, WEBOGRAPHIE)</t>
+  </si>
+  <si>
+    <t>Rapport (structure ,intorduction,2	ANALYSE 2.1	Planification de toutes les tâches à réaliser Planification des tâches (outil GitHub Projects))</t>
   </si>
 </sst>
 </file>
@@ -1268,7 +1271,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>8.3333333333333329E-2</c:v>
+                  <c:v>0.10069444444444445</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>2.0833333333333332E-2</c:v>
@@ -2240,7 +2243,7 @@
       </c>
       <c r="C3" s="22" t="str">
         <f>INT(E4/1440)&amp;" jours "&amp;INT(MOD(E4/1440,1)*24)&amp;" heurs "&amp;INT(MOD(MOD(E4/1440,1)*24,1)*60)&amp;" minutes"</f>
-        <v>0 jours 18 heurs 30 minutes</v>
+        <v>0 jours 18 heurs 54 minutes</v>
       </c>
       <c r="D3" s="22"/>
       <c r="E3" s="3"/>
@@ -2259,11 +2262,11 @@
       </c>
       <c r="D4" s="22">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>870</v>
+        <v>895</v>
       </c>
       <c r="E4" s="40">
         <f>SUM(C4:D4)</f>
-        <v>1110</v>
+        <v>1135</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="7"/>
@@ -3246,15 +3249,23 @@
       <c r="G47" s="56"/>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A48" s="8" t="str">
+      <c r="A48" s="8">
         <f>IF(ISBLANK(B48),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B48))</f>
-        <v/>
-      </c>
-      <c r="B48" s="46"/>
+        <v>21</v>
+      </c>
+      <c r="B48" s="46">
+        <v>45797</v>
+      </c>
       <c r="C48" s="47"/>
-      <c r="D48" s="48"/>
-      <c r="E48" s="49"/>
-      <c r="F48" s="35"/>
+      <c r="D48" s="48">
+        <v>25</v>
+      </c>
+      <c r="E48" s="49" t="s">
+        <v>6</v>
+      </c>
+      <c r="F48" s="35" t="s">
+        <v>83</v>
+      </c>
       <c r="G48" s="55"/>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
@@ -9202,7 +9213,7 @@
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Analyse!C7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>120</v>
+        <v>145</v>
       </c>
       <c r="C7" s="27" t="str">
         <f>'Journal de travail'!M11</f>
@@ -9210,7 +9221,7 @@
       </c>
       <c r="D7" s="33">
         <f t="shared" si="0"/>
-        <v>8.3333333333333329E-2</v>
+        <v>0.10069444444444445</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
@@ -9291,7 +9302,7 @@
       </c>
       <c r="D12" s="34">
         <f>SUM(D4:D11)</f>
-        <v>0.77083333333333337</v>
+        <v>0.78819444444444442</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Rapprot + "uploads" folder + diagram.png
</commit_message>
<xml_diff>
--- a/documentation/JDT-personal/Journal-de-Travail_NademoYosef.xlsx
+++ b/documentation/JDT-personal/Journal-de-Travail_NademoYosef.xlsx
@@ -8,10 +8,10 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pn25kdv\Documents\GitHub\Passion_lecture_FRONTEND\documentation\JDT-personal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{116E6EBC-87C9-4839-A4C7-8D10508DE0FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8950711-7612-4635-9233-F0593F2212C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="Mvap2W10CJFFJsnvkGXSiMLvpngxTMJbJsIKFe7Hzjn0XDcmjGuvBC2FjUCZ/hpRpUhUrG1T4kBlDAIo3yqmSQ==" workbookSaltValue="KXjgXOcsUZI/j7UgPKltzw==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="3960" yWindow="540" windowWidth="23520" windowHeight="14235" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
+    <workbookView xWindow="29535" yWindow="0" windowWidth="23520" windowHeight="15600" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal de travail" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="88">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -321,6 +321,20 @@
   </si>
   <si>
     <t>Rapport (structure ,intorduction,2	ANALYSE 2.1	Planification de toutes les tâches à réaliser Planification des tâches (outil GitHub Projects))</t>
+  </si>
+  <si>
+    <t>ANALYSE :Planification des tâches (outil GitHub Projects)</t>
+  </si>
+  <si>
+    <t>Réalisation (sécurité, fonctionnalités techniques, gestion Git/GitHub).</t>
+  </si>
+  <si>
+    <t>Schéma de l’architecture représentant les interactions entre le
+frontend et le backend tout en situant les différents composants (API
+REST, la base de données, l’ORM, etc)</t>
+  </si>
+  <si>
+    <t>diagram.png</t>
   </si>
 </sst>
 </file>
@@ -1271,7 +1285,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.10069444444444445</c:v>
+                  <c:v>0.1423611111111111</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>2.0833333333333332E-2</c:v>
@@ -2243,7 +2257,7 @@
       </c>
       <c r="C3" s="22" t="str">
         <f>INT(E4/1440)&amp;" jours "&amp;INT(MOD(E4/1440,1)*24)&amp;" heurs "&amp;INT(MOD(MOD(E4/1440,1)*24,1)*60)&amp;" minutes"</f>
-        <v>0 jours 18 heurs 54 minutes</v>
+        <v>0 jours 19 heurs 55 minutes</v>
       </c>
       <c r="D3" s="22"/>
       <c r="E3" s="3"/>
@@ -2262,11 +2276,11 @@
       </c>
       <c r="D4" s="22">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>895</v>
+        <v>955</v>
       </c>
       <c r="E4" s="40">
         <f>SUM(C4:D4)</f>
-        <v>1135</v>
+        <v>1195</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="7"/>
@@ -3269,40 +3283,66 @@
       <c r="G48" s="55"/>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A49" s="16" t="str">
+      <c r="A49" s="16">
         <f>IF(ISBLANK(B49),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B49))</f>
-        <v/>
-      </c>
-      <c r="B49" s="50"/>
+        <v>22</v>
+      </c>
+      <c r="B49" s="50">
+        <v>45804</v>
+      </c>
       <c r="C49" s="51"/>
-      <c r="D49" s="52"/>
-      <c r="E49" s="53"/>
-      <c r="F49" s="35"/>
+      <c r="D49" s="52">
+        <v>10</v>
+      </c>
+      <c r="E49" s="53" t="s">
+        <v>6</v>
+      </c>
+      <c r="F49" s="35" t="s">
+        <v>84</v>
+      </c>
       <c r="G49" s="56"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A50" s="8" t="str">
+      <c r="A50" s="8">
         <f>IF(ISBLANK(B50),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B50))</f>
-        <v/>
-      </c>
-      <c r="B50" s="46"/>
+        <v>22</v>
+      </c>
+      <c r="B50" s="46">
+        <v>45804</v>
+      </c>
       <c r="C50" s="47"/>
-      <c r="D50" s="48"/>
-      <c r="E50" s="49"/>
-      <c r="F50" s="35"/>
+      <c r="D50" s="48">
+        <v>25</v>
+      </c>
+      <c r="E50" s="49" t="s">
+        <v>6</v>
+      </c>
+      <c r="F50" s="35" t="s">
+        <v>85</v>
+      </c>
       <c r="G50" s="55"/>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A51" s="16" t="str">
+    <row r="51" spans="1:7" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="A51" s="16">
         <f>IF(ISBLANK(B51),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B51))</f>
-        <v/>
-      </c>
-      <c r="B51" s="50"/>
+        <v>22</v>
+      </c>
+      <c r="B51" s="50">
+        <v>45804</v>
+      </c>
       <c r="C51" s="51"/>
-      <c r="D51" s="52"/>
-      <c r="E51" s="53"/>
-      <c r="F51" s="35"/>
-      <c r="G51" s="56"/>
+      <c r="D51" s="52">
+        <v>25</v>
+      </c>
+      <c r="E51" s="53" t="s">
+        <v>6</v>
+      </c>
+      <c r="F51" s="36" t="s">
+        <v>86</v>
+      </c>
+      <c r="G51" s="56" t="s">
+        <v>87</v>
+      </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="8" t="str">
@@ -9213,7 +9253,7 @@
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Analyse!C7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>145</v>
+        <v>205</v>
       </c>
       <c r="C7" s="27" t="str">
         <f>'Journal de travail'!M11</f>
@@ -9221,7 +9261,7 @@
       </c>
       <c r="D7" s="33">
         <f t="shared" si="0"/>
-        <v>0.10069444444444445</v>
+        <v>0.1423611111111111</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
@@ -9302,7 +9342,7 @@
       </c>
       <c r="D12" s="34">
         <f>SUM(D4:D11)</f>
-        <v>0.78819444444444442</v>
+        <v>0.82986111111111105</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
@@ -9325,6 +9365,17 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="be0d3259-a7ce-4623-88ec-81594dfcbc1c" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="99ffe1f3-7857-457f-add0-5bdef636f38d">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D4F20F00DBE2EE49BE9523363A2DF18B" ma:contentTypeVersion="13" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="313dbdbec26224d1c2bb7e3c488b2a4e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="99ffe1f3-7857-457f-add0-5bdef636f38d" xmlns:ns3="be0d3259-a7ce-4623-88ec-81594dfcbc1c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4739345e3d2c6be79c5ae1a54d02a4a7" ns2:_="" ns3:_="">
     <xsd:import namespace="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
@@ -9547,17 +9598,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="be0d3259-a7ce-4623-88ec-81594dfcbc1c" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="99ffe1f3-7857-457f-add0-5bdef636f38d">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>
@@ -9567,6 +9607,17 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="be0d3259-a7ce-4623-88ec-81594dfcbc1c"/>
+    <ds:schemaRef ds:uri="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F2FB702A-DCBD-43A8-A34C-6000FD8861AD}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -9583,15 +9634,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="be0d3259-a7ce-4623-88ec-81594dfcbc1c"/>
-    <ds:schemaRef ds:uri="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
chore(2.3 Analyse de la structure du code qui sera effectuée)
</commit_message>
<xml_diff>
--- a/documentation/JDT-personal/Journal-de-Travail_NademoYosef.xlsx
+++ b/documentation/JDT-personal/Journal-de-Travail_NademoYosef.xlsx
@@ -8,10 +8,10 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pn25kdv\Documents\GitHub\Passion_lecture_FRONTEND\documentation\JDT-personal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF7CC97D-22DF-40A1-ADAE-BE21EABBB4BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99718D96-543A-40B3-8852-9E1279AA1E38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="Mvap2W10CJFFJsnvkGXSiMLvpngxTMJbJsIKFe7Hzjn0XDcmjGuvBC2FjUCZ/hpRpUhUrG1T4kBlDAIo3yqmSQ==" workbookSaltValue="KXjgXOcsUZI/j7UgPKltzw==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="29535" yWindow="525" windowWidth="23520" windowHeight="14235" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal de travail" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="94">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -350,6 +350,9 @@
   </si>
   <si>
     <t>evaluation avec prof, verification d'application</t>
+  </si>
+  <si>
+    <t>2.3 Analyse de la structure du code qui sera effectuée</t>
   </si>
 </sst>
 </file>
@@ -1300,7 +1303,7 @@
                   <c:v>1.3888888888888888E-2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.15972222222222221</c:v>
+                  <c:v>0.1875</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>3.8194444444444448E-2</c:v>
@@ -2272,7 +2275,7 @@
       </c>
       <c r="C3" s="22" t="str">
         <f>INT(E4/1440)&amp;" jours "&amp;INT(MOD(E4/1440,1)*24)&amp;" heurs "&amp;INT(MOD(MOD(E4/1440,1)*24,1)*60)&amp;" minutes"</f>
-        <v>0 jours 21 heurs 45 minutes</v>
+        <v>0 jours 22 heurs 25 minutes</v>
       </c>
       <c r="D3" s="22"/>
       <c r="E3" s="3"/>
@@ -2291,11 +2294,11 @@
       </c>
       <c r="D4" s="22">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>1065</v>
+        <v>1105</v>
       </c>
       <c r="E4" s="40">
         <f>SUM(C4:D4)</f>
-        <v>1305</v>
+        <v>1345</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="7"/>
@@ -3466,16 +3469,24 @@
       <c r="G57" s="56"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A58" s="8" t="str">
+      <c r="A58" s="8">
         <f>IF(ISBLANK(B58),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B58))</f>
-        <v/>
-      </c>
-      <c r="B58" s="46"/>
+        <v>22</v>
+      </c>
+      <c r="B58" s="46">
+        <v>45805</v>
+      </c>
       <c r="C58" s="47"/>
-      <c r="D58" s="48"/>
-      <c r="E58" s="49"/>
+      <c r="D58" s="48">
+        <v>40</v>
+      </c>
+      <c r="E58" s="49" t="s">
+        <v>6</v>
+      </c>
       <c r="F58" s="15"/>
-      <c r="G58" s="55"/>
+      <c r="G58" s="55" t="s">
+        <v>93</v>
+      </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="16" t="str">
@@ -9302,7 +9313,7 @@
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Analyse!C7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>230</v>
+        <v>270</v>
       </c>
       <c r="C7" s="27" t="str">
         <f>'Journal de travail'!M11</f>
@@ -9310,7 +9321,7 @@
       </c>
       <c r="D7" s="33">
         <f t="shared" si="0"/>
-        <v>0.15972222222222221</v>
+        <v>0.1875</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
@@ -9391,7 +9402,7 @@
       </c>
       <c r="D12" s="34">
         <f>SUM(D4:D11)</f>
-        <v>0.90624999999999989</v>
+        <v>0.93402777777777768</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
@@ -9414,6 +9425,17 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="be0d3259-a7ce-4623-88ec-81594dfcbc1c" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="99ffe1f3-7857-457f-add0-5bdef636f38d">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D4F20F00DBE2EE49BE9523363A2DF18B" ma:contentTypeVersion="13" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="313dbdbec26224d1c2bb7e3c488b2a4e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="99ffe1f3-7857-457f-add0-5bdef636f38d" xmlns:ns3="be0d3259-a7ce-4623-88ec-81594dfcbc1c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4739345e3d2c6be79c5ae1a54d02a4a7" ns2:_="" ns3:_="">
     <xsd:import namespace="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
@@ -9636,17 +9658,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="be0d3259-a7ce-4623-88ec-81594dfcbc1c" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="99ffe1f3-7857-457f-add0-5bdef636f38d">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>
@@ -9656,6 +9667,17 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="be0d3259-a7ce-4623-88ec-81594dfcbc1c"/>
+    <ds:schemaRef ds:uri="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F2FB702A-DCBD-43A8-A34C-6000FD8861AD}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -9672,15 +9694,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="be0d3259-a7ce-4623-88ec-81594dfcbc1c"/>
-    <ds:schemaRef ds:uri="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>